<commit_message>
Isi RAB: harga LCD dan nipple, step-down & komponen pasif 0, catatan ganti ESP32-C3 Mini
</commit_message>
<xml_diff>
--- a/anggaran/RAB-alat-praktikum-rev08.xlsx
+++ b/anggaran/RAB-alat-praktikum-rev08.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GunturS\Projec_Ibah\anggaran\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33050906-EA6B-4D13-815E-EE005F0B6C62}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72121C97-3152-46C9-B303-E14EB47B03F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -112,9 +112,6 @@
     <t>Belum</t>
   </si>
   <si>
-    <t>Uno clone ± Rp85 rb kalau ingin lebih mudah dirakit</t>
-  </si>
-  <si>
     <t>LCD 20×4 + modul I2C</t>
   </si>
   <si>
@@ -989,6 +986,9 @@
   </si>
   <si>
     <t>https://shopee.co.id/MAXPUMP-Pompa-Celup-Air-Bersih-DC-12V-24V-Submersible-Pump-Pompa-Kolam-Ikan-Brushless-5m-Aquarium-Hidroponik-i.17799491.12107841427?extraParams=%7B%22display_model_id%22%3A227492409707%2C%22model_selection_logic%22%3A3%7D</t>
+  </si>
+  <si>
+    <t>ganti esp C3 mini</t>
   </si>
 </sst>
 </file>
@@ -1206,8 +1206,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1217,6 +1215,8 @@
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1535,7 +1535,7 @@
     <col min="10" max="10" width="15" customWidth="1"/>
     <col min="11" max="12" width="14" customWidth="1"/>
     <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="24" style="33" customWidth="1"/>
+    <col min="14" max="14" width="24" style="31" customWidth="1"/>
     <col min="15" max="15" width="11" customWidth="1"/>
     <col min="16" max="16" width="40" customWidth="1"/>
   </cols>
@@ -1606,24 +1606,24 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32"/>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32"/>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32"/>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="32"/>
-      <c r="M6" s="32"/>
-      <c r="N6" s="32"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="32"/>
+      <c r="B6" s="35"/>
+      <c r="C6" s="35"/>
+      <c r="D6" s="35"/>
+      <c r="E6" s="35"/>
+      <c r="F6" s="35"/>
+      <c r="G6" s="35"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="35"/>
+      <c r="J6" s="35"/>
+      <c r="K6" s="35"/>
+      <c r="L6" s="35"/>
+      <c r="M6" s="35"/>
+      <c r="N6" s="35"/>
+      <c r="O6" s="35"/>
+      <c r="P6" s="35"/>
     </row>
     <row r="7" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
@@ -1674,7 +1674,7 @@
         <v>25</v>
       </c>
       <c r="P7" s="5" t="s">
-        <v>26</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -1682,13 +1682,13 @@
         <v>2</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>28</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>23</v>
@@ -1706,18 +1706,20 @@
         <f t="shared" si="0"/>
         <v>75000</v>
       </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v/>
+      <c r="J8" s="8">
+        <v>150000</v>
+      </c>
+      <c r="K8" s="7">
+        <f>IF(J8="","",G8*J8)</f>
+        <v>150000</v>
       </c>
       <c r="L8" s="7">
         <f t="shared" si="2"/>
+        <v>150000</v>
+      </c>
+      <c r="M8" s="7">
+        <f t="shared" si="3"/>
         <v>75000</v>
-      </c>
-      <c r="M8" s="7" t="str">
-        <f t="shared" si="3"/>
-        <v/>
       </c>
       <c r="N8" s="9"/>
       <c r="O8" s="6" t="s">
@@ -1730,13 +1732,13 @@
         <v>3</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>31</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>32</v>
       </c>
       <c r="E9" s="4" t="s">
         <v>23</v>
@@ -1772,7 +1774,7 @@
         <v>25</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -1780,13 +1782,13 @@
         <v>4</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>35</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>36</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>23</v>
@@ -1822,7 +1824,7 @@
         <v>25</v>
       </c>
       <c r="P10" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="43.2" x14ac:dyDescent="0.3">
@@ -1830,13 +1832,13 @@
         <v>5</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>40</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>23</v>
@@ -1867,14 +1869,14 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="N11" s="35" t="s">
-        <v>318</v>
+      <c r="N11" s="33" t="s">
+        <v>317</v>
       </c>
       <c r="O11" s="6" t="s">
         <v>25</v>
       </c>
       <c r="P11" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -1882,13 +1884,13 @@
         <v>6</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>44</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>23</v>
@@ -1924,7 +1926,7 @@
         <v>25</v>
       </c>
       <c r="P12" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
@@ -1932,13 +1934,13 @@
         <v>7</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>47</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>48</v>
       </c>
       <c r="E13" s="4" t="s">
         <v>23</v>
@@ -1956,18 +1958,20 @@
         <f t="shared" si="0"/>
         <v>12000</v>
       </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="7" t="str">
+      <c r="J13" s="8">
+        <v>0</v>
+      </c>
+      <c r="K13" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L13" s="7">
         <f t="shared" si="2"/>
-        <v>12000</v>
-      </c>
-      <c r="M13" s="7" t="str">
+        <v>0</v>
+      </c>
+      <c r="M13" s="7">
         <f t="shared" si="3"/>
-        <v/>
+        <v>-12000</v>
       </c>
       <c r="N13" s="9"/>
       <c r="O13" s="6" t="s">
@@ -1980,13 +1984,13 @@
         <v>8</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="E14" s="4" t="s">
         <v>23</v>
@@ -2024,7 +2028,7 @@
         <v>25</v>
       </c>
       <c r="P14" s="5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
@@ -2032,19 +2036,19 @@
         <v>9</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" s="4" t="s">
         <v>55</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>56</v>
       </c>
       <c r="G15" s="6">
         <v>1</v>
@@ -2080,13 +2084,13 @@
         <v>10</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>59</v>
       </c>
       <c r="E16" s="4" t="s">
         <v>23</v>
@@ -2128,13 +2132,13 @@
         <v>11</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>61</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>62</v>
       </c>
       <c r="E17" s="4" t="s">
         <v>23</v>
@@ -2176,13 +2180,13 @@
         <v>12</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="E18" s="4" t="s">
         <v>23</v>
@@ -2224,13 +2228,13 @@
         <v>13</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>67</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="E19" s="4" t="s">
         <v>23</v>
@@ -2272,11 +2276,11 @@
         <v>14</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C20" s="5"/>
       <c r="D20" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E20" s="4" t="s">
         <v>23</v>
@@ -2318,19 +2322,19 @@
         <v>15</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>73</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>74</v>
       </c>
       <c r="G21" s="6">
         <v>1</v>
@@ -2342,18 +2346,20 @@
         <f t="shared" si="0"/>
         <v>15000</v>
       </c>
-      <c r="J21" s="8"/>
-      <c r="K21" s="7" t="str">
+      <c r="J21" s="8">
+        <v>0</v>
+      </c>
+      <c r="K21" s="7">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="L21" s="7">
         <f t="shared" si="2"/>
-        <v>15000</v>
-      </c>
-      <c r="M21" s="7" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" s="7">
         <f t="shared" si="3"/>
-        <v/>
+        <v>-15000</v>
       </c>
       <c r="N21" s="9"/>
       <c r="O21" s="6" t="s">
@@ -2366,19 +2372,19 @@
         <v>16</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D22" s="5" t="s">
-        <v>77</v>
-      </c>
       <c r="E22" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G22" s="6">
         <v>1</v>
@@ -2414,19 +2420,19 @@
         <v>17</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>80</v>
-      </c>
       <c r="E23" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G23" s="6">
         <v>1</v>
@@ -2456,7 +2462,7 @@
         <v>25</v>
       </c>
       <c r="P23" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
@@ -2464,13 +2470,13 @@
         <v>18</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>84</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>23</v>
@@ -2512,16 +2518,16 @@
         <v>19</v>
       </c>
       <c r="B25" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="4" t="s">
         <v>87</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>88</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>24</v>
@@ -2554,7 +2560,7 @@
         <v>25</v>
       </c>
       <c r="P25" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.3">
@@ -2562,16 +2568,16 @@
         <v>20</v>
       </c>
       <c r="B26" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="4" t="s">
         <v>92</v>
-      </c>
-      <c r="E26" s="4" t="s">
-        <v>93</v>
       </c>
       <c r="F26" s="4" t="s">
         <v>24</v>
@@ -2604,7 +2610,7 @@
         <v>25</v>
       </c>
       <c r="P26" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.3">
@@ -2612,16 +2618,16 @@
         <v>21</v>
       </c>
       <c r="B27" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="D27" s="5" t="s">
-        <v>97</v>
-      </c>
       <c r="E27" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F27" s="4" t="s">
         <v>24</v>
@@ -2654,7 +2660,7 @@
         <v>25</v>
       </c>
       <c r="P27" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.3">
@@ -2662,14 +2668,14 @@
         <v>22</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C28" s="5"/>
       <c r="D28" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F28" s="4" t="s">
         <v>24</v>
@@ -2702,13 +2708,13 @@
         <v>25</v>
       </c>
       <c r="P28" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A29" s="11"/>
       <c r="B29" s="11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C29" s="11"/>
       <c r="D29" s="11"/>
@@ -2723,49 +2729,49 @@
       <c r="J29" s="11"/>
       <c r="K29" s="12">
         <f>SUMIFS(K7:K28,E7:E28,"Inti")</f>
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="L29" s="12">
         <f>SUMIFS(L7:L28,E7:E28,"Inti")</f>
-        <v>450000</v>
+        <v>498000</v>
       </c>
       <c r="M29" s="11"/>
-      <c r="N29" s="34"/>
+      <c r="N29" s="32"/>
       <c r="O29" s="11"/>
       <c r="P29" s="11"/>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A31" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="B31" s="32"/>
-      <c r="C31" s="32"/>
-      <c r="D31" s="32"/>
-      <c r="E31" s="32"/>
-      <c r="F31" s="32"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="32"/>
-      <c r="J31" s="32"/>
-      <c r="K31" s="32"/>
-      <c r="L31" s="32"/>
-      <c r="M31" s="32"/>
-      <c r="N31" s="32"/>
-      <c r="O31" s="32"/>
-      <c r="P31" s="32"/>
+      <c r="A31" s="34" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="35"/>
+      <c r="C31" s="35"/>
+      <c r="D31" s="35"/>
+      <c r="E31" s="35"/>
+      <c r="F31" s="35"/>
+      <c r="G31" s="35"/>
+      <c r="H31" s="35"/>
+      <c r="I31" s="35"/>
+      <c r="J31" s="35"/>
+      <c r="K31" s="35"/>
+      <c r="L31" s="35"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
+      <c r="O31" s="35"/>
+      <c r="P31" s="35"/>
     </row>
     <row r="32" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A32" s="4">
         <v>23</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="D32" s="5" t="s">
         <v>105</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>106</v>
       </c>
       <c r="E32" s="4" t="s">
         <v>23</v>
@@ -2801,7 +2807,7 @@
         <v>25</v>
       </c>
       <c r="P32" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.3">
@@ -2809,13 +2815,13 @@
         <v>24</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="D33" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>110</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>23</v>
@@ -2857,13 +2863,13 @@
         <v>25</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="D34" s="5" t="s">
         <v>112</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>113</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>23</v>
@@ -2905,19 +2911,19 @@
         <v>26</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C35" s="5" t="s">
+      <c r="D35" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="E35" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F35" s="4" t="s">
         <v>116</v>
-      </c>
-      <c r="E35" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>117</v>
       </c>
       <c r="G35" s="6">
         <v>2</v>
@@ -2947,7 +2953,7 @@
         <v>25</v>
       </c>
       <c r="P35" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -2955,13 +2961,13 @@
         <v>27</v>
       </c>
       <c r="B36" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="C36" s="5" t="s">
+      <c r="D36" s="5" t="s">
         <v>120</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>121</v>
       </c>
       <c r="E36" s="4" t="s">
         <v>23</v>
@@ -2997,7 +3003,7 @@
         <v>25</v>
       </c>
       <c r="P36" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -3005,13 +3011,13 @@
         <v>28</v>
       </c>
       <c r="B37" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="D37" s="5" t="s">
         <v>124</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>125</v>
       </c>
       <c r="E37" s="4" t="s">
         <v>23</v>
@@ -3047,7 +3053,7 @@
         <v>25</v>
       </c>
       <c r="P37" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -3055,11 +3061,11 @@
         <v>29</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C38" s="5"/>
       <c r="D38" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>23</v>
@@ -3101,19 +3107,19 @@
         <v>30</v>
       </c>
       <c r="B39" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C39" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="D39" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>131</v>
-      </c>
       <c r="E39" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G39" s="6">
         <v>1</v>
@@ -3149,19 +3155,19 @@
         <v>31</v>
       </c>
       <c r="B40" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C40" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D40" s="5" t="s">
-        <v>134</v>
-      </c>
       <c r="E40" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G40" s="6">
         <v>1</v>
@@ -3197,13 +3203,13 @@
         <v>32</v>
       </c>
       <c r="B41" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C41" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="D41" s="5" t="s">
         <v>136</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>137</v>
       </c>
       <c r="E41" s="4" t="s">
         <v>23</v>
@@ -3245,13 +3251,13 @@
         <v>33</v>
       </c>
       <c r="B42" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="C42" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="D42" s="5" t="s">
         <v>139</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>140</v>
       </c>
       <c r="E42" s="4" t="s">
         <v>23</v>
@@ -3293,13 +3299,13 @@
         <v>34</v>
       </c>
       <c r="B43" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C43" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="D43" s="5" t="s">
         <v>142</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>143</v>
       </c>
       <c r="E43" s="4" t="s">
         <v>23</v>
@@ -3335,7 +3341,7 @@
         <v>25</v>
       </c>
       <c r="P43" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -3343,13 +3349,13 @@
         <v>35</v>
       </c>
       <c r="B44" s="5" t="s">
+        <v>144</v>
+      </c>
+      <c r="C44" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="D44" s="5" t="s">
         <v>146</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>147</v>
       </c>
       <c r="E44" s="4" t="s">
         <v>23</v>
@@ -3391,11 +3397,11 @@
         <v>36</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C45" s="5"/>
       <c r="D45" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E45" s="4" t="s">
         <v>23</v>
@@ -3437,13 +3443,13 @@
         <v>37</v>
       </c>
       <c r="B46" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C46" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="C46" s="5" t="s">
+      <c r="D46" s="5" t="s">
         <v>151</v>
-      </c>
-      <c r="D46" s="5" t="s">
-        <v>152</v>
       </c>
       <c r="E46" s="4" t="s">
         <v>23</v>
@@ -3479,7 +3485,7 @@
         <v>25</v>
       </c>
       <c r="P46" s="5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.3">
@@ -3487,19 +3493,19 @@
         <v>38</v>
       </c>
       <c r="B47" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C47" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="C47" s="5" t="s">
+      <c r="D47" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D47" s="5" t="s">
+      <c r="E47" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F47" s="4" t="s">
         <v>156</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F47" s="4" t="s">
-        <v>157</v>
       </c>
       <c r="G47" s="6">
         <v>6</v>
@@ -3535,13 +3541,13 @@
         <v>39</v>
       </c>
       <c r="B48" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="C48" s="5" t="s">
+      <c r="D48" s="5" t="s">
         <v>159</v>
-      </c>
-      <c r="D48" s="5" t="s">
-        <v>160</v>
       </c>
       <c r="E48" s="4" t="s">
         <v>23</v>
@@ -3559,25 +3565,27 @@
         <f t="shared" si="4"/>
         <v>32000</v>
       </c>
-      <c r="J48" s="8"/>
-      <c r="K48" s="7" t="str">
-        <f t="shared" si="5"/>
-        <v/>
+      <c r="J48" s="8">
+        <v>30000</v>
+      </c>
+      <c r="K48" s="7">
+        <f>IF(J48="","",G48*J48)</f>
+        <v>120000</v>
       </c>
       <c r="L48" s="7">
         <f t="shared" si="6"/>
-        <v>32000</v>
-      </c>
-      <c r="M48" s="7" t="str">
+        <v>120000</v>
+      </c>
+      <c r="M48" s="7">
         <f t="shared" si="7"/>
-        <v/>
+        <v>88000</v>
       </c>
       <c r="N48" s="9"/>
       <c r="O48" s="6" t="s">
         <v>25</v>
       </c>
       <c r="P48" s="5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.3">
@@ -3585,13 +3593,13 @@
         <v>40</v>
       </c>
       <c r="B49" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="C49" s="5" t="s">
+      <c r="D49" s="5" t="s">
         <v>163</v>
-      </c>
-      <c r="D49" s="5" t="s">
-        <v>164</v>
       </c>
       <c r="E49" s="4" t="s">
         <v>23</v>
@@ -3633,13 +3641,13 @@
         <v>41</v>
       </c>
       <c r="B50" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="D50" s="5" t="s">
         <v>166</v>
-      </c>
-      <c r="D50" s="5" t="s">
-        <v>167</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>23</v>
@@ -3681,19 +3689,19 @@
         <v>42</v>
       </c>
       <c r="B51" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C51" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="D51" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="D51" s="5" t="s">
-        <v>170</v>
-      </c>
       <c r="E51" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G51" s="6">
         <v>1</v>
@@ -3729,19 +3737,19 @@
         <v>43</v>
       </c>
       <c r="B52" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="C52" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="D52" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D52" s="5" t="s">
-        <v>173</v>
-      </c>
       <c r="E52" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G52" s="6">
         <v>1</v>
@@ -3777,16 +3785,16 @@
         <v>44</v>
       </c>
       <c r="B53" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="5" t="s">
         <v>174</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="D53" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="D53" s="5" t="s">
-        <v>176</v>
-      </c>
       <c r="E53" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>24</v>
@@ -3825,16 +3833,16 @@
         <v>45</v>
       </c>
       <c r="B54" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="C54" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="D54" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="D54" s="5" t="s">
-        <v>179</v>
-      </c>
       <c r="E54" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F54" s="4" t="s">
         <v>24</v>
@@ -3867,7 +3875,7 @@
         <v>25</v>
       </c>
       <c r="P54" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="55" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
@@ -3875,16 +3883,16 @@
         <v>46</v>
       </c>
       <c r="B55" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="C55" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="D55" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="D55" s="5" t="s">
-        <v>183</v>
-      </c>
       <c r="E55" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F55" s="4" t="s">
         <v>24</v>
@@ -3921,7 +3929,7 @@
     <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A56" s="11"/>
       <c r="B56" s="11" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C56" s="11"/>
       <c r="D56" s="11"/>
@@ -3936,49 +3944,49 @@
       <c r="J56" s="11"/>
       <c r="K56" s="12">
         <f>SUMIFS(K32:K55,E32:E55,"Inti")</f>
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="L56" s="12">
         <f>SUMIFS(L32:L55,E32:E55,"Inti")</f>
-        <v>1024000</v>
+        <v>1112000</v>
       </c>
       <c r="M56" s="11"/>
-      <c r="N56" s="34"/>
+      <c r="N56" s="32"/>
       <c r="O56" s="11"/>
       <c r="P56" s="11"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A58" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="B58" s="32"/>
-      <c r="C58" s="32"/>
-      <c r="D58" s="32"/>
-      <c r="E58" s="32"/>
-      <c r="F58" s="32"/>
-      <c r="G58" s="32"/>
-      <c r="H58" s="32"/>
-      <c r="I58" s="32"/>
-      <c r="J58" s="32"/>
-      <c r="K58" s="32"/>
-      <c r="L58" s="32"/>
-      <c r="M58" s="32"/>
-      <c r="N58" s="32"/>
-      <c r="O58" s="32"/>
-      <c r="P58" s="32"/>
+      <c r="A58" s="34" t="s">
+        <v>184</v>
+      </c>
+      <c r="B58" s="35"/>
+      <c r="C58" s="35"/>
+      <c r="D58" s="35"/>
+      <c r="E58" s="35"/>
+      <c r="F58" s="35"/>
+      <c r="G58" s="35"/>
+      <c r="H58" s="35"/>
+      <c r="I58" s="35"/>
+      <c r="J58" s="35"/>
+      <c r="K58" s="35"/>
+      <c r="L58" s="35"/>
+      <c r="M58" s="35"/>
+      <c r="N58" s="35"/>
+      <c r="O58" s="35"/>
+      <c r="P58" s="35"/>
     </row>
     <row r="59" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
         <v>47</v>
       </c>
       <c r="B59" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C59" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="C59" s="5" t="s">
+      <c r="D59" s="5" t="s">
         <v>187</v>
-      </c>
-      <c r="D59" s="5" t="s">
-        <v>188</v>
       </c>
       <c r="E59" s="4" t="s">
         <v>23</v>
@@ -4020,19 +4028,19 @@
         <v>48</v>
       </c>
       <c r="B60" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C60" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="D60" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="D60" s="5" t="s">
-        <v>191</v>
-      </c>
       <c r="E60" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G60" s="6">
         <v>3</v>
@@ -4068,13 +4076,13 @@
         <v>49</v>
       </c>
       <c r="B61" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C61" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="C61" s="5" t="s">
+      <c r="D61" s="5" t="s">
         <v>193</v>
-      </c>
-      <c r="D61" s="5" t="s">
-        <v>194</v>
       </c>
       <c r="E61" s="4" t="s">
         <v>23</v>
@@ -4116,19 +4124,19 @@
         <v>50</v>
       </c>
       <c r="B62" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="C62" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="C62" s="5" t="s">
+      <c r="D62" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="E62" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F62" s="4" t="s">
         <v>197</v>
-      </c>
-      <c r="E62" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F62" s="4" t="s">
-        <v>198</v>
       </c>
       <c r="G62" s="6">
         <v>1</v>
@@ -4164,13 +4172,13 @@
         <v>51</v>
       </c>
       <c r="B63" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C63" s="5" t="s">
         <v>199</v>
       </c>
-      <c r="C63" s="5" t="s">
+      <c r="D63" s="5" t="s">
         <v>200</v>
-      </c>
-      <c r="D63" s="5" t="s">
-        <v>201</v>
       </c>
       <c r="E63" s="4" t="s">
         <v>23</v>
@@ -4212,13 +4220,13 @@
         <v>52</v>
       </c>
       <c r="B64" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="C64" s="5" t="s">
         <v>202</v>
       </c>
-      <c r="C64" s="5" t="s">
+      <c r="D64" s="5" t="s">
         <v>203</v>
-      </c>
-      <c r="D64" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="E64" s="4" t="s">
         <v>23</v>
@@ -4260,19 +4268,19 @@
         <v>53</v>
       </c>
       <c r="B65" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="C65" s="5" t="s">
         <v>205</v>
       </c>
-      <c r="C65" s="5" t="s">
+      <c r="D65" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D65" s="5" t="s">
-        <v>207</v>
-      </c>
       <c r="E65" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G65" s="6">
         <v>1</v>
@@ -4308,11 +4316,11 @@
         <v>54</v>
       </c>
       <c r="B66" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C66" s="5"/>
       <c r="D66" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E66" s="4" t="s">
         <v>23</v>
@@ -4352,7 +4360,7 @@
     <row r="67" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A67" s="11"/>
       <c r="B67" s="11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C67" s="11"/>
       <c r="D67" s="11"/>
@@ -4374,40 +4382,40 @@
         <v>362000</v>
       </c>
       <c r="M67" s="11"/>
-      <c r="N67" s="34"/>
+      <c r="N67" s="32"/>
       <c r="O67" s="11"/>
       <c r="P67" s="11"/>
     </row>
     <row r="69" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A69" s="31" t="s">
-        <v>211</v>
-      </c>
-      <c r="B69" s="32"/>
-      <c r="C69" s="32"/>
-      <c r="D69" s="32"/>
-      <c r="E69" s="32"/>
-      <c r="F69" s="32"/>
-      <c r="G69" s="32"/>
-      <c r="H69" s="32"/>
-      <c r="I69" s="32"/>
-      <c r="J69" s="32"/>
-      <c r="K69" s="32"/>
-      <c r="L69" s="32"/>
-      <c r="M69" s="32"/>
-      <c r="N69" s="32"/>
-      <c r="O69" s="32"/>
-      <c r="P69" s="32"/>
+      <c r="A69" s="34" t="s">
+        <v>210</v>
+      </c>
+      <c r="B69" s="35"/>
+      <c r="C69" s="35"/>
+      <c r="D69" s="35"/>
+      <c r="E69" s="35"/>
+      <c r="F69" s="35"/>
+      <c r="G69" s="35"/>
+      <c r="H69" s="35"/>
+      <c r="I69" s="35"/>
+      <c r="J69" s="35"/>
+      <c r="K69" s="35"/>
+      <c r="L69" s="35"/>
+      <c r="M69" s="35"/>
+      <c r="N69" s="35"/>
+      <c r="O69" s="35"/>
+      <c r="P69" s="35"/>
     </row>
     <row r="70" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A70" s="4">
         <v>55</v>
       </c>
       <c r="B70" s="5" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C70" s="5"/>
       <c r="D70" s="5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="E70" s="4" t="s">
         <v>23</v>
@@ -4449,11 +4457,11 @@
         <v>56</v>
       </c>
       <c r="B71" s="5" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C71" s="5"/>
       <c r="D71" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="E71" s="4" t="s">
         <v>23</v>
@@ -4495,13 +4503,13 @@
         <v>57</v>
       </c>
       <c r="B72" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="C72" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="C72" s="5" t="s">
+      <c r="D72" s="5" t="s">
         <v>217</v>
-      </c>
-      <c r="D72" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="E72" s="4" t="s">
         <v>23</v>
@@ -4543,17 +4551,17 @@
         <v>58</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C73" s="5"/>
       <c r="D73" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="E73" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F73" s="4" t="s">
         <v>220</v>
-      </c>
-      <c r="E73" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F73" s="4" t="s">
-        <v>221</v>
       </c>
       <c r="G73" s="6">
         <v>2</v>
@@ -4589,19 +4597,19 @@
         <v>59</v>
       </c>
       <c r="B74" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="C74" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="C74" s="5" t="s">
+      <c r="D74" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D74" s="5" t="s">
+      <c r="E74" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F74" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="E74" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F74" s="4" t="s">
-        <v>225</v>
       </c>
       <c r="G74" s="6">
         <v>1</v>
@@ -4631,7 +4639,7 @@
         <v>25</v>
       </c>
       <c r="P74" s="5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="75" spans="1:16" x14ac:dyDescent="0.3">
@@ -4639,17 +4647,17 @@
         <v>60</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C75" s="5"/>
       <c r="D75" s="5" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E75" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G75" s="6">
         <v>1</v>
@@ -4683,7 +4691,7 @@
     <row r="76" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A76" s="11"/>
       <c r="B76" s="11" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C76" s="11"/>
       <c r="D76" s="11"/>
@@ -4705,42 +4713,42 @@
         <v>96000</v>
       </c>
       <c r="M76" s="11"/>
-      <c r="N76" s="34"/>
+      <c r="N76" s="32"/>
       <c r="O76" s="11"/>
       <c r="P76" s="11"/>
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A78" s="31" t="s">
-        <v>230</v>
-      </c>
-      <c r="B78" s="32"/>
-      <c r="C78" s="32"/>
-      <c r="D78" s="32"/>
-      <c r="E78" s="32"/>
-      <c r="F78" s="32"/>
-      <c r="G78" s="32"/>
-      <c r="H78" s="32"/>
-      <c r="I78" s="32"/>
-      <c r="J78" s="32"/>
-      <c r="K78" s="32"/>
-      <c r="L78" s="32"/>
-      <c r="M78" s="32"/>
-      <c r="N78" s="32"/>
-      <c r="O78" s="32"/>
-      <c r="P78" s="32"/>
+      <c r="A78" s="34" t="s">
+        <v>229</v>
+      </c>
+      <c r="B78" s="35"/>
+      <c r="C78" s="35"/>
+      <c r="D78" s="35"/>
+      <c r="E78" s="35"/>
+      <c r="F78" s="35"/>
+      <c r="G78" s="35"/>
+      <c r="H78" s="35"/>
+      <c r="I78" s="35"/>
+      <c r="J78" s="35"/>
+      <c r="K78" s="35"/>
+      <c r="L78" s="35"/>
+      <c r="M78" s="35"/>
+      <c r="N78" s="35"/>
+      <c r="O78" s="35"/>
+      <c r="P78" s="35"/>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A79" s="4">
         <v>61</v>
       </c>
       <c r="B79" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="C79" s="5" t="s">
         <v>231</v>
       </c>
-      <c r="C79" s="5" t="s">
+      <c r="D79" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="D79" s="5" t="s">
-        <v>233</v>
       </c>
       <c r="E79" s="4" t="s">
         <v>23</v>
@@ -4776,7 +4784,7 @@
         <v>25</v>
       </c>
       <c r="P79" s="5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.3">
@@ -4784,19 +4792,19 @@
         <v>62</v>
       </c>
       <c r="B80" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="C80" s="5" t="s">
         <v>235</v>
       </c>
-      <c r="C80" s="5" t="s">
+      <c r="D80" s="5" t="s">
         <v>236</v>
       </c>
-      <c r="D80" s="5" t="s">
-        <v>237</v>
-      </c>
       <c r="E80" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G80" s="6">
         <v>1</v>
@@ -4826,7 +4834,7 @@
         <v>25</v>
       </c>
       <c r="P80" s="5" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.3">
@@ -4834,13 +4842,13 @@
         <v>63</v>
       </c>
       <c r="B81" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="C81" s="5" t="s">
         <v>239</v>
       </c>
-      <c r="C81" s="5" t="s">
+      <c r="D81" s="5" t="s">
         <v>240</v>
-      </c>
-      <c r="D81" s="5" t="s">
-        <v>241</v>
       </c>
       <c r="E81" s="4" t="s">
         <v>23</v>
@@ -4876,7 +4884,7 @@
         <v>25</v>
       </c>
       <c r="P81" s="5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.3">
@@ -4884,11 +4892,11 @@
         <v>64</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="C82" s="5"/>
       <c r="D82" s="5" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E82" s="4" t="s">
         <v>23</v>
@@ -4930,11 +4938,11 @@
         <v>65</v>
       </c>
       <c r="B83" s="5" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C83" s="5"/>
       <c r="D83" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="E83" s="4" t="s">
         <v>23</v>
@@ -4974,7 +4982,7 @@
     <row r="84" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A84" s="11"/>
       <c r="B84" s="11" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C84" s="11"/>
       <c r="D84" s="11"/>
@@ -4996,46 +5004,46 @@
         <v>195000</v>
       </c>
       <c r="M84" s="11"/>
-      <c r="N84" s="34"/>
+      <c r="N84" s="32"/>
       <c r="O84" s="11"/>
       <c r="P84" s="11"/>
     </row>
     <row r="86" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A86" s="31" t="s">
-        <v>248</v>
-      </c>
-      <c r="B86" s="32"/>
-      <c r="C86" s="32"/>
-      <c r="D86" s="32"/>
-      <c r="E86" s="32"/>
-      <c r="F86" s="32"/>
-      <c r="G86" s="32"/>
-      <c r="H86" s="32"/>
-      <c r="I86" s="32"/>
-      <c r="J86" s="32"/>
-      <c r="K86" s="32"/>
-      <c r="L86" s="32"/>
-      <c r="M86" s="32"/>
-      <c r="N86" s="32"/>
-      <c r="O86" s="32"/>
-      <c r="P86" s="32"/>
+      <c r="A86" s="34" t="s">
+        <v>247</v>
+      </c>
+      <c r="B86" s="35"/>
+      <c r="C86" s="35"/>
+      <c r="D86" s="35"/>
+      <c r="E86" s="35"/>
+      <c r="F86" s="35"/>
+      <c r="G86" s="35"/>
+      <c r="H86" s="35"/>
+      <c r="I86" s="35"/>
+      <c r="J86" s="35"/>
+      <c r="K86" s="35"/>
+      <c r="L86" s="35"/>
+      <c r="M86" s="35"/>
+      <c r="N86" s="35"/>
+      <c r="O86" s="35"/>
+      <c r="P86" s="35"/>
     </row>
     <row r="87" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
         <v>66</v>
       </c>
       <c r="B87" s="5" t="s">
+        <v>248</v>
+      </c>
+      <c r="C87" s="5" t="s">
         <v>249</v>
-      </c>
-      <c r="C87" s="5" t="s">
-        <v>250</v>
       </c>
       <c r="D87" s="5"/>
       <c r="E87" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G87" s="6">
         <v>1</v>
@@ -5065,7 +5073,7 @@
         <v>25</v>
       </c>
       <c r="P87" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="88" spans="1:16" x14ac:dyDescent="0.3">
@@ -5073,17 +5081,17 @@
         <v>67</v>
       </c>
       <c r="B88" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="C88" s="5" t="s">
         <v>252</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>253</v>
       </c>
       <c r="D88" s="5"/>
       <c r="E88" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G88" s="6">
         <v>1</v>
@@ -5117,7 +5125,7 @@
     <row r="89" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A89" s="11"/>
       <c r="B89" s="11" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C89" s="11"/>
       <c r="D89" s="11"/>
@@ -5139,46 +5147,46 @@
         <v>150000</v>
       </c>
       <c r="M89" s="11"/>
-      <c r="N89" s="34"/>
+      <c r="N89" s="32"/>
       <c r="O89" s="11"/>
       <c r="P89" s="11"/>
     </row>
     <row r="91" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A91" s="31" t="s">
-        <v>255</v>
-      </c>
-      <c r="B91" s="32"/>
-      <c r="C91" s="32"/>
-      <c r="D91" s="32"/>
-      <c r="E91" s="32"/>
-      <c r="F91" s="32"/>
-      <c r="G91" s="32"/>
-      <c r="H91" s="32"/>
-      <c r="I91" s="32"/>
-      <c r="J91" s="32"/>
-      <c r="K91" s="32"/>
-      <c r="L91" s="32"/>
-      <c r="M91" s="32"/>
-      <c r="N91" s="32"/>
-      <c r="O91" s="32"/>
-      <c r="P91" s="32"/>
+      <c r="A91" s="34" t="s">
+        <v>254</v>
+      </c>
+      <c r="B91" s="35"/>
+      <c r="C91" s="35"/>
+      <c r="D91" s="35"/>
+      <c r="E91" s="35"/>
+      <c r="F91" s="35"/>
+      <c r="G91" s="35"/>
+      <c r="H91" s="35"/>
+      <c r="I91" s="35"/>
+      <c r="J91" s="35"/>
+      <c r="K91" s="35"/>
+      <c r="L91" s="35"/>
+      <c r="M91" s="35"/>
+      <c r="N91" s="35"/>
+      <c r="O91" s="35"/>
+      <c r="P91" s="35"/>
     </row>
     <row r="92" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A92" s="4">
         <v>68</v>
       </c>
       <c r="B92" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="C92" s="5" t="s">
         <v>256</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>257</v>
       </c>
       <c r="D92" s="5"/>
       <c r="E92" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G92" s="6">
         <v>1</v>
@@ -5214,17 +5222,17 @@
         <v>69</v>
       </c>
       <c r="B93" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="C93" s="5" t="s">
         <v>258</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>259</v>
       </c>
       <c r="D93" s="5"/>
       <c r="E93" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G93" s="6">
         <v>1</v>
@@ -5260,17 +5268,17 @@
         <v>70</v>
       </c>
       <c r="B94" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="C94" s="5" t="s">
         <v>260</v>
-      </c>
-      <c r="C94" s="5" t="s">
-        <v>261</v>
       </c>
       <c r="D94" s="5"/>
       <c r="E94" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G94" s="6">
         <v>1</v>
@@ -5306,17 +5314,17 @@
         <v>71</v>
       </c>
       <c r="B95" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="C95" s="5" t="s">
         <v>262</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>263</v>
       </c>
       <c r="D95" s="5"/>
       <c r="E95" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G95" s="6">
         <v>1</v>
@@ -5352,17 +5360,17 @@
         <v>72</v>
       </c>
       <c r="B96" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="C96" s="5" t="s">
         <v>264</v>
-      </c>
-      <c r="C96" s="5" t="s">
-        <v>265</v>
       </c>
       <c r="D96" s="5"/>
       <c r="E96" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G96" s="6">
         <v>1</v>
@@ -5398,17 +5406,17 @@
         <v>73</v>
       </c>
       <c r="B97" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="C97" s="5" t="s">
         <v>266</v>
-      </c>
-      <c r="C97" s="5" t="s">
-        <v>267</v>
       </c>
       <c r="D97" s="5"/>
       <c r="E97" s="4" t="s">
         <v>23</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G97" s="6">
         <v>1</v>
@@ -5438,7 +5446,7 @@
         <v>25</v>
       </c>
       <c r="P97" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="98" spans="1:16" x14ac:dyDescent="0.3">
@@ -5446,17 +5454,17 @@
         <v>74</v>
       </c>
       <c r="B98" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="C98" s="5" t="s">
         <v>269</v>
-      </c>
-      <c r="C98" s="5" t="s">
-        <v>270</v>
       </c>
       <c r="D98" s="5"/>
       <c r="E98" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G98" s="6">
         <v>1</v>
@@ -5490,7 +5498,7 @@
     <row r="99" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A99" s="11"/>
       <c r="B99" s="11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C99" s="11"/>
       <c r="D99" s="11"/>
@@ -5512,7 +5520,7 @@
         <v>1500000</v>
       </c>
       <c r="M99" s="11"/>
-      <c r="N99" s="34"/>
+      <c r="N99" s="32"/>
       <c r="O99" s="11"/>
       <c r="P99" s="11"/>
     </row>
@@ -5556,17 +5564,17 @@
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="15" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="B4" s="16">
         <v>2000000</v>
@@ -5577,7 +5585,7 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="15" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="B5" s="17">
         <v>0.1</v>
@@ -5595,7 +5603,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="18" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
@@ -5604,24 +5612,24 @@
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="B8" s="19" t="s">
         <v>277</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="C8" s="19" t="s">
         <v>278</v>
       </c>
-      <c r="C8" s="19" t="s">
+      <c r="D8" s="19" t="s">
         <v>279</v>
       </c>
-      <c r="D8" s="19" t="s">
+      <c r="E8" s="19" t="s">
         <v>280</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B9" s="21">
         <f>SUMIFS(RAB!$I$7:$I$28,RAB!$E$7:$E$28,"Inti")</f>
@@ -5629,20 +5637,20 @@
       </c>
       <c r="C9" s="21">
         <f>SUMIFS(RAB!$K$7:$K$28,RAB!$E$7:$E$28,"Inti")</f>
-        <v>0</v>
+        <v>150000</v>
       </c>
       <c r="D9" s="21">
         <f>SUMIFS(RAB!$L$7:$L$28,RAB!$E$7:$E$28,"Inti")</f>
-        <v>450000</v>
+        <v>498000</v>
       </c>
       <c r="E9" s="20" t="str">
         <f>COUNTIFS(RAB!$E$7:$E$28,"Inti",RAB!$J$7:$J$28,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$7:$E$28,"Inti")</f>
-        <v>2 / 18</v>
+        <v>5 / 18</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="20" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B10" s="21">
         <f>SUMIFS(RAB!$I$32:$I$55,RAB!$E$32:$E$55,"Inti")</f>
@@ -5650,20 +5658,20 @@
       </c>
       <c r="C10" s="21">
         <f>SUMIFS(RAB!$K$32:$K$55,RAB!$E$32:$E$55,"Inti")</f>
-        <v>0</v>
+        <v>120000</v>
       </c>
       <c r="D10" s="21">
         <f>SUMIFS(RAB!$L$32:$L$55,RAB!$E$32:$E$55,"Inti")</f>
-        <v>1024000</v>
+        <v>1112000</v>
       </c>
       <c r="E10" s="20" t="str">
         <f>COUNTIFS(RAB!$E$32:$E$55,"Inti",RAB!$J$32:$J$55,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$32:$E$55,"Inti")</f>
-        <v>0 / 20</v>
+        <v>1 / 20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B11" s="21">
         <f>SUMIFS(RAB!$I$59:$I$66,RAB!$E$59:$E$66,"Inti")</f>
@@ -5684,7 +5692,7 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="20" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="B12" s="21">
         <f>SUMIFS(RAB!$I$70:$I$75,RAB!$E$70:$E$75,"Inti")</f>
@@ -5705,7 +5713,7 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="20" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="B13" s="21">
         <f>SUMIFS(RAB!$I$79:$I$83,RAB!$E$79:$E$83,"Inti")</f>
@@ -5726,7 +5734,7 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="22" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="B14" s="23">
         <f>SUM(B9:B13)</f>
@@ -5734,17 +5742,17 @@
       </c>
       <c r="C14" s="23">
         <f>SUM(C9:C13)</f>
-        <v>0</v>
+        <v>270000</v>
       </c>
       <c r="D14" s="23">
         <f>SUM(D9:D13)</f>
-        <v>2127000</v>
+        <v>2263000</v>
       </c>
       <c r="E14" s="22"/>
     </row>
     <row r="15" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A15" s="20" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="B15" s="21">
         <f>B14*$B$5</f>
@@ -5753,15 +5761,15 @@
       <c r="C15" s="21"/>
       <c r="D15" s="21">
         <f>D14*$B$5</f>
-        <v>212700</v>
+        <v>226300</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="20" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="B16" s="21">
         <f>SUMIFS(RAB!$I$87:$I$88,RAB!$E$87:$E$88,"Inti")</f>
@@ -5779,7 +5787,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="22" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B17" s="23">
         <f>B14+B15+B16</f>
@@ -5788,13 +5796,13 @@
       <c r="C17" s="23"/>
       <c r="D17" s="23">
         <f>D14+D15+D16</f>
-        <v>2489700</v>
+        <v>2639300</v>
       </c>
       <c r="E17" s="22"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="20" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="B18" s="21">
         <f>SUMIFS(RAB!$I$92:$I$98,RAB!$E$92:$E$98,"Inti")</f>
@@ -5809,7 +5817,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="24" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="B19" s="25">
         <f>B17+B18</f>
@@ -5818,13 +5826,13 @@
       <c r="C19" s="25"/>
       <c r="D19" s="25">
         <f>D17+D18</f>
-        <v>3989700</v>
+        <v>4139300</v>
       </c>
       <c r="E19" s="24"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="26" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B20" s="27">
         <f>B19-$B$4</f>
@@ -5833,7 +5841,7 @@
       <c r="C20" s="27"/>
       <c r="D20" s="27">
         <f>D19-$B$4</f>
-        <v>1989700</v>
+        <v>2139300</v>
       </c>
       <c r="E20" s="26"/>
     </row>
@@ -5854,7 +5862,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="20" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B22" s="28">
         <f>B18/B19</f>
@@ -5863,7 +5871,7 @@
       <c r="C22" s="21"/>
       <c r="D22" s="28">
         <f>D18/D19</f>
-        <v>0.3759681179036018</v>
+        <v>0.36238011257942165</v>
       </c>
       <c r="E22" s="20"/>
     </row>
@@ -5876,7 +5884,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="18" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -5885,24 +5893,24 @@
     </row>
     <row r="25" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="19" t="s">
+        <v>276</v>
+      </c>
+      <c r="B25" s="19" t="s">
         <v>277</v>
       </c>
-      <c r="B25" s="19" t="s">
+      <c r="C25" s="19" t="s">
         <v>278</v>
       </c>
-      <c r="C25" s="19" t="s">
+      <c r="D25" s="19" t="s">
         <v>279</v>
       </c>
-      <c r="D25" s="19" t="s">
-        <v>280</v>
-      </c>
       <c r="E25" s="19" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A26" s="20" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B26" s="21">
         <f>SUMIFS(RAB!$I$6:$I$100,RAB!$E$6:$E$100,"Lengkap")+(SUMIFS(RAB!$I$6:$I$100,RAB!$E$6:$E$100,"Lengkap")-SUMIFS(RAB!$I$92:$I$98,RAB!$E$92:$E$98,"Lengkap"))*$B$5</f>
@@ -5917,12 +5925,12 @@
         <v>365000</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A27" s="24" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="B27" s="25">
         <f>B19+B26</f>
@@ -5931,15 +5939,15 @@
       <c r="C27" s="25"/>
       <c r="D27" s="25">
         <f>D19+D26</f>
-        <v>4354700</v>
+        <v>4504300</v>
       </c>
       <c r="E27" s="24" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A28" s="20" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="B28" s="21">
         <f>SUMIFS(RAB!$I$6:$I$100,RAB!$E$6:$E$100,"Opsional")</f>
@@ -5954,7 +5962,7 @@
         <v>345000</v>
       </c>
       <c r="E28" s="20" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>
@@ -5972,42 +5980,42 @@
   <sheetData>
     <row r="1" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" s="29" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="30" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" s="30" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" s="30" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" s="30" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="30" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" s="30" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="8" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="30" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
@@ -6015,32 +6023,32 @@
     </row>
     <row r="10" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="29" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" s="30" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" s="30" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" s="30" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="14" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A14" s="30" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="30" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
RAB: ganti MCU ke ESP32-C3 Super Mini, tambah level shifter, MOSFET 3,3 V, dan buck pompa
</commit_message>
<xml_diff>
--- a/anggaran/RAB-alat-praktikum-rev08.xlsx
+++ b/anggaran/RAB-alat-praktikum-rev08.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RAB'!$A$5:$P$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RAB'!$A$5:$P$102</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'RAB'!$5:$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -577,7 +577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P99"/>
+  <dimension ref="A1:P101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -720,17 +720,17 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Arduino Nano (clone CH340)</t>
+          <t>ESP32-C3 Super Mini</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>ATmega328P, 5 V</t>
+          <t>RISC-V 160 MHz, WiFi/BLE, USB-C, logika 3,3 V</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Otak alat: baca S1, kontrol PI pompa, layar, tombol</t>
+          <t>Otak alat: baca S1, kontrol PI pompa, layar, tombol, log data</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -744,18 +744,16 @@
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>50000</v>
+        <v>40000</v>
       </c>
       <c r="I7" s="8">
         <f>G7*H7</f>
         <v/>
       </c>
-      <c r="J7" s="9" t="n">
-        <v>0</v>
-      </c>
+      <c r="J7" s="9" t="n"/>
       <c r="K7" s="8">
         <f>IF(J7="","",G7*J7)</f>
         <v/>
@@ -776,7 +774,7 @@
       </c>
       <c r="P7" s="6" t="inlineStr">
         <is>
-          <t>ganti esp C3 mini</t>
+          <t>1 cadangan. Pin tidak tahan 5 V; jangan pakai GPIO 2/8/9 untuk kendali pompa</t>
         </is>
       </c>
     </row>
@@ -1044,17 +1042,17 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Modul MOSFET logic-level</t>
+          <t>MOSFET gate 3,3 V</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>D4184 / IRLZ44N, ≥ 5 A</t>
+          <t>AO3400 / IRLML6244 (atau modul + transistor pendorong), ≥ 3 A</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Driver PWM pompa</t>
+          <t>Saklar PWM pompa / kendali buck</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -1068,10 +1066,10 @@
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H12" s="8" t="n">
-        <v>15000</v>
+        <v>7500</v>
       </c>
       <c r="I12" s="8">
         <f>G12*H12</f>
@@ -1108,17 +1106,17 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Modul step-down 12 V → 5 V</t>
+          <t>Modul buck DC-DC 5 A (pompa)</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>LM2596 / Mini-360</t>
+          <t>XL4015 / setara, tegangan keluaran bisa diatur</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Catu daya MCU &amp; LCD</t>
+          <t>Atur kecepatan pompa lewat tegangan (pompa brushless tanpa kabel PWM)</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1135,15 +1133,13 @@
         <v>1</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>12000</v>
+        <v>30000</v>
       </c>
       <c r="I13" s="8">
         <f>G13*H13</f>
         <v/>
       </c>
-      <c r="J13" s="9" t="n">
-        <v>0</v>
-      </c>
+      <c r="J13" s="9" t="n"/>
       <c r="K13" s="8">
         <f>IF(J13="","",G13*J13)</f>
         <v/>
@@ -1162,7 +1158,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P13" s="6" t="inlineStr"/>
+      <c r="P13" s="6" t="inlineStr">
+        <is>
+          <t>Cara kendali dari MCU ditentukan saat uji bangku</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="n">
@@ -1170,17 +1170,17 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Adaptor 12 V 5 A</t>
+          <t>Level shifter 4 kanal</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Switching, casing tertutup</t>
+          <t>BSS138, 3,3 V ↔ 5 V</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Sumber daya utama</t>
+          <t>Sinyal YF-S201 &amp; I2C LCD ke ESP32-C3</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -1197,15 +1197,13 @@
         <v>1</v>
       </c>
       <c r="H14" s="8" t="n">
-        <v>70000</v>
+        <v>8000</v>
       </c>
       <c r="I14" s="8">
         <f>G14*H14</f>
         <v/>
       </c>
-      <c r="J14" s="9" t="n">
-        <v>0</v>
-      </c>
+      <c r="J14" s="9" t="n"/>
       <c r="K14" s="8">
         <f>IF(J14="","",G14*J14)</f>
         <v/>
@@ -1224,11 +1222,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P14" s="6" t="inlineStr">
-        <is>
-          <t>Letakkan jauh dari air</t>
-        </is>
-      </c>
+      <c r="P14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="n">
@@ -1236,17 +1230,17 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>Sekring + holder inline</t>
+          <t>Modul step-down 12 V → 5 V</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>3–5 A</t>
+          <t>LM2596 / Mini-360</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Proteksi hubung singkat</t>
+          <t>Catu daya MCU &amp; LCD</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -1256,20 +1250,22 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="I15" s="8">
         <f>G15*H15</f>
         <v/>
       </c>
-      <c r="J15" s="9" t="n"/>
+      <c r="J15" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="K15" s="8">
         <f>IF(J15="","",G15*J15)</f>
         <v/>
@@ -1296,17 +1292,17 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Saklar daya (rocker)</t>
+          <t>Adaptor 12 V 5 A</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>6 A</t>
+          <t>Switching, casing tertutup</t>
         </is>
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>ON/OFF alat</t>
+          <t>Sumber daya utama</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1323,13 +1319,15 @@
         <v>1</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>5000</v>
+        <v>70000</v>
       </c>
       <c r="I16" s="8">
         <f>G16*H16</f>
         <v/>
       </c>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="K16" s="8">
         <f>IF(J16="","",G16*J16)</f>
         <v/>
@@ -1348,7 +1346,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P16" s="6" t="inlineStr"/>
+      <c r="P16" s="6" t="inlineStr">
+        <is>
+          <t>Letakkan jauh dari air</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">
@@ -1356,17 +1358,17 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Jack DC panel female</t>
+          <t>Sekring + holder inline</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>5,5 × 2,1 mm</t>
+          <t>3–5 A</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Input adaptor</t>
+          <t>Proteksi hubung singkat</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1376,14 +1378,14 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>5000</v>
+        <v>8000</v>
       </c>
       <c r="I17" s="8">
         <f>G17*H17</f>
@@ -1416,17 +1418,17 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Potensiometer 10 kΩ + knob</t>
+          <t>Saklar daya (rocker)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Linear, dudukan panel</t>
+          <t>6 A</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Kenop target debit</t>
+          <t>ON/OFF alat</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1443,7 +1445,7 @@
         <v>1</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>10000</v>
+        <v>5000</v>
       </c>
       <c r="I18" s="8">
         <f>G18*H18</f>
@@ -1476,17 +1478,17 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Tombol tekan panel</t>
+          <t>Jack DC panel female</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>12 mm, momentary</t>
+          <t>5,5 × 2,1 mm</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Tombol CEK + Start/Stop</t>
+          <t>Input adaptor</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1500,7 +1502,7 @@
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H19" s="8" t="n">
         <v>5000</v>
@@ -1536,13 +1538,17 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Buzzer aktif 5 V</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr"/>
+          <t>Potensiometer 10 kΩ + knob</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>Linear, dudukan panel</t>
+        </is>
+      </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Sonifikasi debit &amp; alarm</t>
+          <t>Kenop target debit</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1559,7 +1565,7 @@
         <v>1</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="I20" s="8">
         <f>G20*H20</f>
@@ -1592,17 +1598,17 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Komponen pasif</t>
+          <t>Tombol tekan panel</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Resistor 10 kΩ &amp; 4,7 kΩ, kapasitor filter, dioda flyback 1N5819</t>
+          <t>12 mm, momentary</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Pull-down gate, pull-up &amp; filter sensor, proteksi pompa</t>
+          <t>Tombol CEK + Start/Stop</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1612,22 +1618,20 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>paket</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H21" s="8" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
       <c r="I21" s="8">
         <f>G21*H21</f>
         <v/>
       </c>
-      <c r="J21" s="9" t="n">
-        <v>0</v>
-      </c>
+      <c r="J21" s="9" t="n"/>
       <c r="K21" s="8">
         <f>IF(J21="","",G21*J21)</f>
         <v/>
@@ -1654,17 +1658,13 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>PCB lubang + header + terminal sekrup</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>± 7 × 9 cm</t>
-        </is>
-      </c>
+          <t>Buzzer aktif 5 V</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr"/>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>Papan rangkaian</t>
+          <t>Sonifikasi debit &amp; alarm</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1674,14 +1674,14 @@
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G22" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>20000</v>
+        <v>5000</v>
       </c>
       <c r="I22" s="8">
         <f>G22*H22</f>
@@ -1714,17 +1714,17 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Kabel &amp; heatshrink</t>
+          <t>Komponen pasif</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Kabel serabut, jumper, kabel sensor berpelindung ± 5 m</t>
+          <t>Resistor 10 kΩ &amp; 4,7 kΩ, kapasitor filter, dioda flyback 1N5819</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Pengkabelan; jalur sensor dipisah dari kabel pompa</t>
+          <t>Pull-down gate, pull-up &amp; filter sensor, proteksi pompa</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1741,13 +1741,15 @@
         <v>1</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="I23" s="8">
         <f>G23*H23</f>
         <v/>
       </c>
-      <c r="J23" s="9" t="n"/>
+      <c r="J23" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="K23" s="8">
         <f>IF(J23="","",G23*J23)</f>
         <v/>
@@ -1766,11 +1768,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P23" s="6" t="inlineStr">
-        <is>
-          <t>Kabel berpelindung mengurangi pulsa palsu dari derau motor</t>
-        </is>
-      </c>
+      <c r="P23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="n">
@@ -1778,17 +1776,17 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>Kotak elektronik tahan cipratan</t>
+          <t>PCB lubang + header + terminal sekrup</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Junction box IP65 ± 15 × 10 × 7 cm</t>
+          <t>± 7 × 9 cm</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Elektronik di atas garis air</t>
+          <t>Papan rangkaian</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1798,14 +1796,14 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G24" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>45000</v>
+        <v>20000</v>
       </c>
       <c r="I24" s="8">
         <f>G24*H24</f>
@@ -1836,36 +1834,36 @@
       <c r="A25" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="11" t="inlineStr">
-        <is>
-          <t>Sensor flow YF-S401 (S2)</t>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Kabel &amp; heatshrink</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>0,3–6 L/min</t>
+          <t>Kabel serabut, jumper, kabel sensor berpelindung ± 5 m</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Sensor kedua di zona C</t>
+          <t>Pengkabelan; jalur sensor dipisah dari kabel pompa</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t>Lengkap</t>
+          <t>Inti</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>paket</t>
         </is>
       </c>
       <c r="G25" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>45000</v>
+        <v>35000</v>
       </c>
       <c r="I25" s="8">
         <f>G25*H25</f>
@@ -1892,7 +1890,7 @@
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>Uji rugi tekanan dulu: harus ≤ ± 90 mm di 6 L/min</t>
+          <t>Kabel berpelindung mengurangi pulsa palsu dari derau motor</t>
         </is>
       </c>
     </row>
@@ -1900,24 +1898,24 @@
       <c r="A26" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B26" s="11" t="inlineStr">
-        <is>
-          <t>Stop kontak / adaptor ber-RCD</t>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>Kotak elektronik tahan cipratan</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Portable RCD 30 mA</t>
+          <t>Junction box IP65 ± 15 × 10 × 7 cm</t>
         </is>
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Keselamatan listrik dekat air</t>
+          <t>Elektronik di atas garis air</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t>Opsional</t>
+          <t>Inti</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
@@ -1929,7 +1927,7 @@
         <v>1</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>200000</v>
+        <v>45000</v>
       </c>
       <c r="I26" s="8">
         <f>G26*H26</f>
@@ -1954,11 +1952,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P26" s="6" t="inlineStr">
-        <is>
-          <t>Tidak perlu jika stop kontak lab sudah ber-RCD</t>
-        </is>
-      </c>
+      <c r="P26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="n">
@@ -1966,22 +1960,22 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Sensor tekanan analog 0–10 kPa</t>
+          <t>Sensor flow YF-S401 (S2)</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>MPX5010DP / XGZP6847</t>
+          <t>0,3–6 L/min</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Demo hidrostatis tangki</t>
+          <t>Sensor kedua di zona C</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>Opsional</t>
+          <t>Lengkap</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1993,7 +1987,7 @@
         <v>1</v>
       </c>
       <c r="H27" s="8" t="n">
-        <v>120000</v>
+        <v>45000</v>
       </c>
       <c r="I27" s="8">
         <f>G27*H27</f>
@@ -2020,7 +2014,7 @@
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>Hanya jika hidrostatis masuk materi skripsi</t>
+          <t>Uji rugi tekanan dulu: harus ≤ ± 90 mm di 6 L/min</t>
         </is>
       </c>
     </row>
@@ -2030,13 +2024,17 @@
       </c>
       <c r="B28" s="11" t="inlineStr">
         <is>
-          <t>Sensor ultrasonik HC-SR04</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr"/>
+          <t>Stop kontak / adaptor ber-RCD</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>Portable RCD 30 mA</t>
+        </is>
+      </c>
       <c r="D28" s="6" t="inlineStr">
         <is>
-          <t>Tinggi air tangki (demo hidrostatis)</t>
+          <t>Keselamatan listrik dekat air</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2053,7 +2051,7 @@
         <v>1</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>15000</v>
+        <v>200000</v>
       </c>
       <c r="I28" s="8">
         <f>G28*H28</f>
@@ -2080,171 +2078,171 @@
       </c>
       <c r="P28" s="6" t="inlineStr">
         <is>
+          <t>Tidak perlu jika stop kontak lab sudah ber-RCD</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Sensor tekanan analog 0–10 kPa</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>MPX5010DP / XGZP6847</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>Demo hidrostatis tangki</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Opsional</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>120000</v>
+      </c>
+      <c r="I29" s="8">
+        <f>G29*H29</f>
+        <v/>
+      </c>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="8">
+        <f>IF(J29="","",G29*J29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="8">
+        <f>IF(J29="",I29,K29)</f>
+        <v/>
+      </c>
+      <c r="M29" s="8">
+        <f>IF(J29="","",K29-I29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="10" t="n"/>
+      <c r="O29" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P29" s="6" t="inlineStr">
+        <is>
+          <t>Hanya jika hidrostatis masuk materi skripsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Sensor ultrasonik HC-SR04</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr"/>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Tinggi air tangki (demo hidrostatis)</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Opsional</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="8" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I30" s="8">
+        <f>G30*H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="9" t="n"/>
+      <c r="K30" s="8">
+        <f>IF(J30="","",G30*J30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="8">
+        <f>IF(J30="",I30,K30)</f>
+        <v/>
+      </c>
+      <c r="M30" s="8">
+        <f>IF(J30="","",K30-I30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="10" t="n"/>
+      <c r="O30" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P30" s="6" t="inlineStr">
+        <is>
           <t>Pasangan sensor tekanan di atas</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="12" t="n"/>
-      <c r="B29" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="12" t="inlineStr">
         <is>
           <t>Subtotal Elektronik — paket inti</t>
         </is>
       </c>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="12" t="n"/>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="12" t="n"/>
-      <c r="I29" s="13">
-        <f>SUMIFS(I7:I28,E7:E28,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J29" s="12" t="n"/>
-      <c r="K29" s="13">
-        <f>SUMIFS(K7:K28,E7:E28,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L29" s="13">
-        <f>SUMIFS(L7:L28,E7:E28,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M29" s="12" t="n"/>
-      <c r="N29" s="12" t="n"/>
-      <c r="O29" s="12" t="n"/>
-      <c r="P29" s="12" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="12" t="n"/>
+      <c r="I31" s="13">
+        <f>SUMIFS(I7:I30,E7:E30,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J31" s="12" t="n"/>
+      <c r="K31" s="13">
+        <f>SUMIFS(K7:K30,E7:E30,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L31" s="13">
+        <f>SUMIFS(L7:L30,E7:E30,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M31" s="12" t="n"/>
+      <c r="N31" s="12" t="n"/>
+      <c r="O31" s="12" t="n"/>
+      <c r="P31" s="12" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>B. MEKANIS — HIDROLIK (pipa, aliran, manometer)</t>
         </is>
       </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="n">
-        <v>23</v>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>Tangki akrilik custom + tutup</t>
-        </is>
-      </c>
-      <c r="C32" s="6" t="inlineStr">
-        <is>
-          <t>± 30 × 20 × 25 cm, tebal 4–5 mm</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="inlineStr">
-        <is>
-          <t>Tangki air tunggal</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H32" s="8" t="n">
-        <v>220000</v>
-      </c>
-      <c r="I32" s="8">
-        <f>G32*H32</f>
-        <v/>
-      </c>
-      <c r="J32" s="9" t="n"/>
-      <c r="K32" s="8">
-        <f>IF(J32="","",G32*J32)</f>
-        <v/>
-      </c>
-      <c r="L32" s="8">
-        <f>IF(J32="",I32,K32)</f>
-        <v/>
-      </c>
-      <c r="M32" s="8">
-        <f>IF(J32="","",K32-I32)</f>
-        <v/>
-      </c>
-      <c r="N32" s="10" t="n"/>
-      <c r="O32" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P32" s="6" t="inlineStr">
-        <is>
-          <t>Alternatif hemat: kontainer plastik bening ± Rp60 rb. Uji bangku pakai ember</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="n">
-        <v>24</v>
-      </c>
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>Sekat tangki</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Potongan akrilik</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Pisahkan air balik dari hisapan pompa</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H33" s="8" t="n">
-        <v>15000</v>
-      </c>
-      <c r="I33" s="8">
-        <f>G33*H33</f>
-        <v/>
-      </c>
-      <c r="J33" s="9" t="n"/>
-      <c r="K33" s="8">
-        <f>IF(J33="","",G33*J33)</f>
-        <v/>
-      </c>
-      <c r="L33" s="8">
-        <f>IF(J33="",I33,K33)</f>
-        <v/>
-      </c>
-      <c r="M33" s="8">
-        <f>IF(J33="","",K33-I33)</f>
-        <v/>
-      </c>
-      <c r="N33" s="10" t="n"/>
-      <c r="O33" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="n">
@@ -2252,17 +2250,17 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>Saringan hisapan pompa</t>
+          <t>Tangki akrilik custom + tutup</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Spons / kasa halus</t>
+          <t>± 30 × 20 × 25 cm, tebal 4–5 mm</t>
         </is>
       </c>
       <c r="D34" s="6" t="inlineStr">
         <is>
-          <t>Cegah serpihan menyumbat S1 &amp; sadap</t>
+          <t>Tangki air tunggal</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -2279,7 +2277,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>10000</v>
+        <v>220000</v>
       </c>
       <c r="I34" s="8">
         <f>G34*H34</f>
@@ -2304,7 +2302,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P34" s="6" t="inlineStr"/>
+      <c r="P34" s="6" t="inlineStr">
+        <is>
+          <t>Alternatif hemat: kontainer plastik bening ± Rp60 rb. Uji bangku pakai ember</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="n">
@@ -2312,17 +2314,17 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>Tabung akrilik OD 25 / ID 19 mm</t>
+          <t>Sekat tangki</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
         <is>
-          <t>Panjang 1 m per batang</t>
+          <t>Potongan akrilik</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Pipa uji: sebelum venturi &amp; tanjakan</t>
+          <t>Pisahkan air balik dari hisapan pompa</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -2332,14 +2334,14 @@
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>batang</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G35" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>75000</v>
+        <v>15000</v>
       </c>
       <c r="I35" s="8">
         <f>G35*H35</f>
@@ -2364,11 +2366,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P35" s="6" t="inlineStr">
-        <is>
-          <t>Ukur ID riil dengan jangka sorong sebelum cetak venturi</t>
-        </is>
-      </c>
+      <c r="P35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="n">
@@ -2376,17 +2374,17 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>Venturi cetak 3D PETG</t>
+          <t>Saringan hisapan pompa</t>
         </is>
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>ID 19 → leher 10 → 19, nipple sadap menyatu</t>
+          <t>Spons / kasa halus</t>
         </is>
       </c>
       <c r="D36" s="6" t="inlineStr">
         <is>
-          <t>Zona A (bukti utama)</t>
+          <t>Cegah serpihan menyumbat S1 &amp; sadap</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -2400,10 +2398,10 @@
         </is>
       </c>
       <c r="G36" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>50000</v>
+        <v>10000</v>
       </c>
       <c r="I36" s="8">
         <f>G36*H36</f>
@@ -2428,11 +2426,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P36" s="6" t="inlineStr">
-        <is>
-          <t>Cetak 3, pakai yang lehernya paling presisi (Δh ∝ d⁻⁴)</t>
-        </is>
-      </c>
+      <c r="P36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="n">
@@ -2440,17 +2434,17 @@
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>Katup searah swing/flapper 3/4"</t>
+          <t>Tabung akrilik OD 25 / ID 19 mm</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>Tekanan buka rendah (bukan tipe pegas)</t>
+          <t>Panjang 1 m per batang</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Tahan air saat pompa mati → uji nol</t>
+          <t>Pipa uji: sebelum venturi &amp; tanjakan</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -2460,14 +2454,14 @@
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>batang</t>
         </is>
       </c>
       <c r="G37" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>50000</v>
+        <v>75000</v>
       </c>
       <c r="I37" s="8">
         <f>G37*H37</f>
@@ -2494,7 +2488,7 @@
       </c>
       <c r="P37" s="6" t="inlineStr">
         <is>
-          <t>Uji bangku: tahan kolom 170 mm ≥ 10 menit</t>
+          <t>Ukur ID riil dengan jangka sorong sebelum cetak venturi</t>
         </is>
       </c>
     </row>
@@ -2504,13 +2498,17 @@
       </c>
       <c r="B38" s="6" t="inlineStr">
         <is>
-          <t>Ball valve PVC 3/4"</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr"/>
+          <t>Venturi cetak 3D PETG</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>ID 19 → leher 10 → 19, nipple sadap menyatu</t>
+        </is>
+      </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>Penyetelan &amp; perawatan (bukan kenop siswa)</t>
+          <t>Zona A (bukti utama)</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -2524,10 +2522,10 @@
         </is>
       </c>
       <c r="G38" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H38" s="8" t="n">
-        <v>15000</v>
+        <v>50000</v>
       </c>
       <c r="I38" s="8">
         <f>G38*H38</f>
@@ -2552,7 +2550,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P38" s="6" t="inlineStr"/>
+      <c r="P38" s="6" t="inlineStr">
+        <is>
+          <t>Cetak 3, pakai yang lehernya paling presisi (Δh ∝ d⁻⁴)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="n">
@@ -2560,17 +2562,17 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>Pipa PVC 3/4" AW</t>
+          <t>Katup searah swing/flapper 3/4"</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>1 batang 4 m</t>
+          <t>Tekanan buka rendah (bukan tipe pegas)</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Leher angsa, pipa balik, pipa limpah</t>
+          <t>Tahan air saat pompa mati → uji nol</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -2580,14 +2582,14 @@
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>batang</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G39" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>45000</v>
+        <v>50000</v>
       </c>
       <c r="I39" s="8">
         <f>G39*H39</f>
@@ -2612,7 +2614,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P39" s="6" t="inlineStr"/>
+      <c r="P39" s="6" t="inlineStr">
+        <is>
+          <t>Uji bangku: tahan kolom 170 mm ≥ 10 menit</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="n">
@@ -2620,17 +2626,13 @@
       </c>
       <c r="B40" s="6" t="inlineStr">
         <is>
-          <t>Fitting PVC 3/4"</t>
-        </is>
-      </c>
-      <c r="C40" s="6" t="inlineStr">
-        <is>
-          <t>Elbow, tee, sok drat (± 10 pcs)</t>
-        </is>
-      </c>
+          <t>Ball valve PVC 3/4"</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr"/>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>Sambungan pipa</t>
+          <t>Penyetelan &amp; perawatan (bukan kenop siswa)</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -2640,14 +2642,14 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>paket</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G40" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H40" s="8" t="n">
-        <v>50000</v>
+        <v>15000</v>
       </c>
       <c r="I40" s="8">
         <f>G40*H40</f>
@@ -2680,17 +2682,17 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>Sok reduksi 3/4" ↔ 1/2"</t>
+          <t>Pipa PVC 3/4" AW</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Ulir dalam 1/2"</t>
+          <t>1 batang 4 m</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Sambung S1 (2) &amp; outlet pompa 1/2" (1)</t>
+          <t>Leher angsa, pipa balik, pipa limpah</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -2700,14 +2702,14 @@
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>batang</t>
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>8000</v>
+        <v>45000</v>
       </c>
       <c r="I41" s="8">
         <f>G41*H41</f>
@@ -2740,17 +2742,17 @@
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>Sambungan akrilik ↔ PVC</t>
+          <t>Fitting PVC 3/4"</t>
         </is>
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>Rubber coupling / sok OD 25 mm</t>
+          <t>Elbow, tee, sok drat (± 10 pcs)</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>Transisi tabung akrilik ke fitting PVC</t>
+          <t>Sambungan pipa</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -2760,14 +2762,14 @@
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>paket</t>
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H42" s="8" t="n">
-        <v>12000</v>
+        <v>50000</v>
       </c>
       <c r="I42" s="8">
         <f>G42*H42</f>
@@ -2800,17 +2802,17 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>Tank connector (bulkhead) 3/4"</t>
+          <t>Sok reduksi 3/4" ↔ 1/2"</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Dengan seal karet</t>
+          <t>Ulir dalam 1/2"</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Keluaran pompa &amp; masuk air balik</t>
+          <t>Sambung S1 (2) &amp; outlet pompa 1/2" (1)</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2824,10 +2826,10 @@
         </is>
       </c>
       <c r="G43" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="I43" s="8">
         <f>G43*H43</f>
@@ -2852,11 +2854,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P43" s="6" t="inlineStr">
-        <is>
-          <t>Air balik masuk dari atas, jauh dari pompa</t>
-        </is>
-      </c>
+      <c r="P43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="5" t="n">
@@ -2864,17 +2862,17 @@
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>Corong plastik</t>
+          <t>Sambungan akrilik ↔ PVC</t>
         </is>
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Ø ± 8 cm</t>
+          <t>Rubber coupling / sok OD 25 mm</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>Penampung air jatuh dari leher angsa (anti sifon)</t>
+          <t>Transisi tabung akrilik ke fitting PVC</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2888,10 +2886,10 @@
         </is>
       </c>
       <c r="G44" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H44" s="8" t="n">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="I44" s="8">
         <f>G44*H44</f>
@@ -2924,13 +2922,17 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>Keran kuras 1/2"</t>
-        </is>
-      </c>
-      <c r="C45" s="6" t="inlineStr"/>
+          <t>Tank connector (bulkhead) 3/4"</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>Dengan seal karet</t>
+        </is>
+      </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Pengurasan tangki (cegah lumut &amp; jentik)</t>
+          <t>Keluaran pompa &amp; masuk air balik</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2944,10 +2946,10 @@
         </is>
       </c>
       <c r="G45" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>15000</v>
+        <v>20000</v>
       </c>
       <c r="I45" s="8">
         <f>G45*H45</f>
@@ -2972,7 +2974,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P45" s="6" t="inlineStr"/>
+      <c r="P45" s="6" t="inlineStr">
+        <is>
+          <t>Air balik masuk dari atas, jauh dari pompa</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="n">
@@ -2980,17 +2986,17 @@
       </c>
       <c r="B46" s="6" t="inlineStr">
         <is>
-          <t>Tabung manometer bening</t>
+          <t>Corong plastik</t>
         </is>
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Akrilik OD 10 / ID 7 mm, 40 cm — satu batch, ID sama</t>
+          <t>Ø ± 8 cm</t>
         </is>
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>Kolom manometer 1–5</t>
+          <t>Penampung air jatuh dari leher angsa (anti sifon)</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -3004,10 +3010,10 @@
         </is>
       </c>
       <c r="G46" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H46" s="8" t="n">
-        <v>15000</v>
+        <v>8000</v>
       </c>
       <c r="I46" s="8">
         <f>G46*H46</f>
@@ -3032,11 +3038,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P46" s="6" t="inlineStr">
-        <is>
-          <t>ID harus identik: beda kapilaritas masuk ke Δh</t>
-        </is>
-      </c>
+      <c r="P46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="5" t="n">
@@ -3044,17 +3046,13 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>Selang bening ID 6 mm</t>
-        </is>
-      </c>
-      <c r="C47" s="6" t="inlineStr">
-        <is>
-          <t>Silikon / PVC</t>
-        </is>
-      </c>
+          <t>Keran kuras 1/2"</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr"/>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Sadap → tabung, pipa limpah panel</t>
+          <t>Pengurasan tangki (cegah lumut &amp; jentik)</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -3064,14 +3062,14 @@
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G47" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>5000</v>
+        <v>15000</v>
       </c>
       <c r="I47" s="8">
         <f>G47*H47</f>
@@ -3104,17 +3102,17 @@
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>Nipple kuningan barb 6 mm</t>
+          <t>Tabung manometer bening</t>
         </is>
       </c>
       <c r="C48" s="6" t="inlineStr">
         <is>
-          <t>Ulir M5 / 1/8"</t>
+          <t>Akrilik OD 10 / ID 7 mm, 40 cm — satu batch, ID sama</t>
         </is>
       </c>
       <c r="D48" s="6" t="inlineStr">
         <is>
-          <t>Titik sadap di tabung akrilik (sadap 1, 3, 4, 5)</t>
+          <t>Kolom manometer 1–5</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -3128,18 +3126,16 @@
         </is>
       </c>
       <c r="G48" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H48" s="8" t="n">
-        <v>8000</v>
+        <v>15000</v>
       </c>
       <c r="I48" s="8">
         <f>G48*H48</f>
         <v/>
       </c>
-      <c r="J48" s="9" t="n">
-        <v>30000</v>
-      </c>
+      <c r="J48" s="9" t="n"/>
       <c r="K48" s="8">
         <f>IF(J48="","",G48*J48)</f>
         <v/>
@@ -3160,7 +3156,7 @@
       </c>
       <c r="P48" s="6" t="inlineStr">
         <is>
-          <t>Sadap 2 sudah menyatu dengan venturi</t>
+          <t>ID harus identik: beda kapilaritas masuk ke Δh</t>
         </is>
       </c>
     </row>
@@ -3170,17 +3166,17 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>Klem penjepit selang</t>
+          <t>Selang bening ID 6 mm</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>Pinch clamp</t>
+          <t>Silikon / PVC</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Buang udara per selang</t>
+          <t>Sadap → tabung, pipa limpah panel</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -3190,14 +3186,14 @@
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G49" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>3000</v>
+        <v>5000</v>
       </c>
       <c r="I49" s="8">
         <f>G49*H49</f>
@@ -3230,17 +3226,17 @@
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>Peredam kolom</t>
+          <t>Nipple kuningan barb 6 mm</t>
         </is>
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>Jarum tumpul 18–20 G / pipa kapiler</t>
+          <t>Ulir M5 / 1/8"</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>Redam getaran kolom akibat pompa</t>
+          <t>Titik sadap di tabung akrilik (sadap 1, 3, 4, 5)</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -3254,16 +3250,18 @@
         </is>
       </c>
       <c r="G50" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H50" s="8" t="n">
-        <v>3000</v>
+        <v>8000</v>
       </c>
       <c r="I50" s="8">
         <f>G50*H50</f>
         <v/>
       </c>
-      <c r="J50" s="9" t="n"/>
+      <c r="J50" s="9" t="n">
+        <v>30000</v>
+      </c>
       <c r="K50" s="8">
         <f>IF(J50="","",G50*J50)</f>
         <v/>
@@ -3282,7 +3280,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P50" s="6" t="inlineStr"/>
+      <c r="P50" s="6" t="inlineStr">
+        <is>
+          <t>Sadap 2 sudah menyatu dengan venturi</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="5" t="n">
@@ -3290,17 +3292,17 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Manifold limpah manometer</t>
+          <t>Klem penjepit selang</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
         <is>
-          <t>Talang di atas tabung + selang ke tangki</t>
+          <t>Pinch clamp</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Air yang meluap kembali ke tangki, tidak ke elektronik</t>
+          <t>Buang udara per selang</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -3310,14 +3312,14 @@
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G51" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H51" s="8" t="n">
-        <v>25000</v>
+        <v>3000</v>
       </c>
       <c r="I51" s="8">
         <f>G51*H51</f>
@@ -3348,36 +3350,36 @@
       <c r="A52" s="5" t="n">
         <v>43</v>
       </c>
-      <c r="B52" s="11" t="inlineStr">
-        <is>
-          <t>Tabung akrilik OD 19 / ID 13 mm</t>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Peredam kolom</t>
         </is>
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>1 m</t>
+          <t>Jarum tumpul 18–20 G / pipa kapiler</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>Pipa zona C</t>
+          <t>Redam getaran kolom akibat pompa</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Lengkap</t>
+          <t>Inti</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>batang</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G52" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H52" s="8" t="n">
-        <v>60000</v>
+        <v>3000</v>
       </c>
       <c r="I52" s="8">
         <f>G52*H52</f>
@@ -3408,36 +3410,36 @@
       <c r="A53" s="5" t="n">
         <v>44</v>
       </c>
-      <c r="B53" s="11" t="inlineStr">
-        <is>
-          <t>Reducer 19 → 13 mm (cetak 3D)</t>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>Manifold limpah manometer</t>
         </is>
       </c>
       <c r="C53" s="6" t="inlineStr">
         <is>
-          <t>Dengan nipple sadap 6</t>
+          <t>Talang di atas tabung + selang ke tangki</t>
         </is>
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Penyempitan zona C</t>
+          <t>Air yang meluap kembali ke tangki, tidak ke elektronik</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
         <is>
-          <t>Lengkap</t>
+          <t>Inti</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G53" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H53" s="8" t="n">
-        <v>30000</v>
+        <v>25000</v>
       </c>
       <c r="I53" s="8">
         <f>G53*H53</f>
@@ -3470,17 +3472,17 @@
       </c>
       <c r="B54" s="11" t="inlineStr">
         <is>
-          <t>Tabung manometer ke-6</t>
+          <t>Tabung akrilik OD 19 / ID 13 mm</t>
         </is>
       </c>
       <c r="C54" s="6" t="inlineStr">
         <is>
-          <t>Sama dengan tabung 1–5</t>
+          <t>1 m</t>
         </is>
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>Kolom zona C / tabung pitot</t>
+          <t>Pipa zona C</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -3490,14 +3492,14 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>batang</t>
         </is>
       </c>
       <c r="G54" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H54" s="8" t="n">
-        <v>15000</v>
+        <v>60000</v>
       </c>
       <c r="I54" s="8">
         <f>G54*H54</f>
@@ -3522,11 +3524,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P54" s="6" t="inlineStr">
-        <is>
-          <t>Bisa juga untuk opsi pitot di paket inti</t>
-        </is>
-      </c>
+      <c r="P54" s="6" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="n">
@@ -3534,22 +3532,22 @@
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Jarum stainless (tabung pitot)</t>
+          <t>Reducer 19 → 13 mm (cetak 3D)</t>
         </is>
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>Ø ± 1,2 mm, dibengkokkan menghadap arus</t>
+          <t>Dengan nipple sadap 6</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Baca energi total di leher venturi</t>
+          <t>Penyempitan zona C</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Opsional</t>
+          <t>Lengkap</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
@@ -3561,7 +3559,7 @@
         <v>1</v>
       </c>
       <c r="H55" s="8" t="n">
-        <v>10000</v>
+        <v>30000</v>
       </c>
       <c r="I55" s="8">
         <f>G55*H55</f>
@@ -3589,162 +3587,166 @@
       <c r="P55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="12" t="n"/>
-      <c r="B56" s="12" t="inlineStr">
+      <c r="A56" s="5" t="n">
+        <v>47</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>Tabung manometer ke-6</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>Sama dengan tabung 1–5</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>Kolom zona C / tabung pitot</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Lengkap</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="8" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I56" s="8">
+        <f>G56*H56</f>
+        <v/>
+      </c>
+      <c r="J56" s="9" t="n"/>
+      <c r="K56" s="8">
+        <f>IF(J56="","",G56*J56)</f>
+        <v/>
+      </c>
+      <c r="L56" s="8">
+        <f>IF(J56="",I56,K56)</f>
+        <v/>
+      </c>
+      <c r="M56" s="8">
+        <f>IF(J56="","",K56-I56)</f>
+        <v/>
+      </c>
+      <c r="N56" s="10" t="n"/>
+      <c r="O56" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P56" s="6" t="inlineStr">
+        <is>
+          <t>Bisa juga untuk opsi pitot di paket inti</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>48</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>Jarum stainless (tabung pitot)</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>Ø ± 1,2 mm, dibengkokkan menghadap arus</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Baca energi total di leher venturi</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Opsional</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I57" s="8">
+        <f>G57*H57</f>
+        <v/>
+      </c>
+      <c r="J57" s="9" t="n"/>
+      <c r="K57" s="8">
+        <f>IF(J57="","",G57*J57)</f>
+        <v/>
+      </c>
+      <c r="L57" s="8">
+        <f>IF(J57="",I57,K57)</f>
+        <v/>
+      </c>
+      <c r="M57" s="8">
+        <f>IF(J57="","",K57-I57)</f>
+        <v/>
+      </c>
+      <c r="N57" s="10" t="n"/>
+      <c r="O57" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P57" s="6" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="12" t="n"/>
+      <c r="B58" s="12" t="inlineStr">
         <is>
           <t>Subtotal Mekanis — Hidrolik — paket inti</t>
         </is>
       </c>
-      <c r="C56" s="12" t="n"/>
-      <c r="D56" s="12" t="n"/>
-      <c r="E56" s="12" t="n"/>
-      <c r="F56" s="12" t="n"/>
-      <c r="G56" s="12" t="n"/>
-      <c r="H56" s="12" t="n"/>
-      <c r="I56" s="13">
-        <f>SUMIFS(I32:I55,E32:E55,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J56" s="12" t="n"/>
-      <c r="K56" s="13">
-        <f>SUMIFS(K32:K55,E32:E55,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L56" s="13">
-        <f>SUMIFS(L32:L55,E32:E55,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M56" s="12" t="n"/>
-      <c r="N56" s="12" t="n"/>
-      <c r="O56" s="12" t="n"/>
-      <c r="P56" s="12" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="C58" s="12" t="n"/>
+      <c r="D58" s="12" t="n"/>
+      <c r="E58" s="12" t="n"/>
+      <c r="F58" s="12" t="n"/>
+      <c r="G58" s="12" t="n"/>
+      <c r="H58" s="12" t="n"/>
+      <c r="I58" s="13">
+        <f>SUMIFS(I34:I57,E34:E57,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J58" s="12" t="n"/>
+      <c r="K58" s="13">
+        <f>SUMIFS(K34:K57,E34:E57,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L58" s="13">
+        <f>SUMIFS(L34:L57,E34:E57,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M58" s="12" t="n"/>
+      <c r="N58" s="12" t="n"/>
+      <c r="O58" s="12" t="n"/>
+      <c r="P58" s="12" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>C. MEKANIS — STRUKTUR &amp; PANEL</t>
         </is>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="n">
-        <v>47</v>
-      </c>
-      <c r="B59" s="6" t="inlineStr">
-        <is>
-          <t>Pelat dasar</t>
-        </is>
-      </c>
-      <c r="C59" s="6" t="inlineStr">
-        <is>
-          <t>Multipleks 18 mm atau akrilik, ± 100 × 35 cm</t>
-        </is>
-      </c>
-      <c r="D59" s="6" t="inlineStr">
-        <is>
-          <t>Alas seluruh alat</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F59" s="5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H59" s="8" t="n">
-        <v>90000</v>
-      </c>
-      <c r="I59" s="8">
-        <f>G59*H59</f>
-        <v/>
-      </c>
-      <c r="J59" s="9" t="n"/>
-      <c r="K59" s="8">
-        <f>IF(J59="","",G59*J59)</f>
-        <v/>
-      </c>
-      <c r="L59" s="8">
-        <f>IF(J59="",I59,K59)</f>
-        <v/>
-      </c>
-      <c r="M59" s="8">
-        <f>IF(J59="","",K59-I59)</f>
-        <v/>
-      </c>
-      <c r="N59" s="10" t="n"/>
-      <c r="O59" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P59" s="6" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="n">
-        <v>48</v>
-      </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>Rangka tegak</t>
-        </is>
-      </c>
-      <c r="C60" s="6" t="inlineStr">
-        <is>
-          <t>Hollow aluminium 20 × 20 mm (atau kayu)</t>
-        </is>
-      </c>
-      <c r="D60" s="6" t="inlineStr">
-        <is>
-          <t>Penyangga pipa &amp; panel</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F60" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="G60" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H60" s="8" t="n">
-        <v>35000</v>
-      </c>
-      <c r="I60" s="8">
-        <f>G60*H60</f>
-        <v/>
-      </c>
-      <c r="J60" s="9" t="n"/>
-      <c r="K60" s="8">
-        <f>IF(J60="","",G60*J60)</f>
-        <v/>
-      </c>
-      <c r="L60" s="8">
-        <f>IF(J60="",I60,K60)</f>
-        <v/>
-      </c>
-      <c r="M60" s="8">
-        <f>IF(J60="","",K60-I60)</f>
-        <v/>
-      </c>
-      <c r="N60" s="10" t="n"/>
-      <c r="O60" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="5" t="n">
@@ -3752,17 +3754,17 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>Papan panel manometer</t>
+          <t>Pelat dasar</t>
         </is>
       </c>
       <c r="C61" s="6" t="inlineStr">
         <is>
-          <t>PVC board / akrilik putih ± 45 × 40 cm</t>
+          <t>Multipleks 18 mm atau akrilik, ± 100 × 35 cm</t>
         </is>
       </c>
       <c r="D61" s="6" t="inlineStr">
         <is>
-          <t>Latar tabung &amp; skala</t>
+          <t>Alas seluruh alat</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -3779,7 +3781,7 @@
         <v>1</v>
       </c>
       <c r="H61" s="8" t="n">
-        <v>50000</v>
+        <v>90000</v>
       </c>
       <c r="I61" s="8">
         <f>G61*H61</f>
@@ -3812,17 +3814,17 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>Cetak stiker skala &amp; peta pipa</t>
+          <t>Rangka tegak</t>
         </is>
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Vinyl: skala 0–350 mm, garis merah z, skala kedua, kode warna</t>
+          <t>Hollow aluminium 20 × 20 mm (atau kayu)</t>
         </is>
       </c>
       <c r="D62" s="6" t="inlineStr">
         <is>
-          <t>Skala baca &amp; petunjuk untuk siswa</t>
+          <t>Penyangga pipa &amp; panel</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -3832,14 +3834,14 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>lembar</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G62" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H62" s="8" t="n">
-        <v>30000</v>
+        <v>35000</v>
       </c>
       <c r="I62" s="8">
         <f>G62*H62</f>
@@ -3872,17 +3874,17 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>Klem pipa (saddle / U-clamp)</t>
+          <t>Papan panel manometer</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>3/4" &amp; 25 mm</t>
+          <t>PVC board / akrilik putih ± 45 × 40 cm</t>
         </is>
       </c>
       <c r="D63" s="6" t="inlineStr">
         <is>
-          <t>Tahan pipa ke rangka</t>
+          <t>Latar tabung &amp; skala</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -3896,10 +3898,10 @@
         </is>
       </c>
       <c r="G63" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H63" s="8" t="n">
-        <v>2500</v>
+        <v>50000</v>
       </c>
       <c r="I63" s="8">
         <f>G63*H63</f>
@@ -3932,17 +3934,17 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>Klip tabung manometer</t>
+          <t>Cetak stiker skala &amp; peta pipa</t>
         </is>
       </c>
       <c r="C64" s="6" t="inlineStr">
         <is>
-          <t>Clip 10 mm</t>
+          <t>Vinyl: skala 0–350 mm, garis merah z, skala kedua, kode warna</t>
         </is>
       </c>
       <c r="D64" s="6" t="inlineStr">
         <is>
-          <t>Tahan tabung di panel</t>
+          <t>Skala baca &amp; petunjuk untuk siswa</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -3952,14 +3954,14 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>lembar</t>
         </is>
       </c>
       <c r="G64" s="7" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H64" s="8" t="n">
-        <v>1500</v>
+        <v>30000</v>
       </c>
       <c r="I64" s="8">
         <f>G64*H64</f>
@@ -3992,17 +3994,17 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Baut, mur, sekrup, siku</t>
+          <t>Klem pipa (saddle / U-clamp)</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>Paket campur</t>
+          <t>3/4" &amp; 25 mm</t>
         </is>
       </c>
       <c r="D65" s="6" t="inlineStr">
         <is>
-          <t>Perakitan rangka &amp; panel</t>
+          <t>Tahan pipa ke rangka</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -4012,14 +4014,14 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>paket</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G65" s="7" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="H65" s="8" t="n">
-        <v>35000</v>
+        <v>2500</v>
       </c>
       <c r="I65" s="8">
         <f>G65*H65</f>
@@ -4052,13 +4054,17 @@
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>Kaki karet</t>
-        </is>
-      </c>
-      <c r="C66" s="6" t="inlineStr"/>
+          <t>Klip tabung manometer</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>Clip 10 mm</t>
+        </is>
+      </c>
       <c r="D66" s="6" t="inlineStr">
         <is>
-          <t>Stabil &amp; anti gores</t>
+          <t>Tahan tabung di panel</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -4072,10 +4078,10 @@
         </is>
       </c>
       <c r="G66" s="7" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H66" s="8" t="n">
-        <v>3000</v>
+        <v>1500</v>
       </c>
       <c r="I66" s="8">
         <f>G66*H66</f>
@@ -4103,154 +4109,158 @@
       <c r="P66" s="6" t="inlineStr"/>
     </row>
     <row r="67">
-      <c r="A67" s="12" t="n"/>
-      <c r="B67" s="12" t="inlineStr">
+      <c r="A67" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>Baut, mur, sekrup, siku</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Paket campur</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Perakitan rangka &amp; panel</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>paket</t>
+        </is>
+      </c>
+      <c r="G67" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" s="8" t="n">
+        <v>35000</v>
+      </c>
+      <c r="I67" s="8">
+        <f>G67*H67</f>
+        <v/>
+      </c>
+      <c r="J67" s="9" t="n"/>
+      <c r="K67" s="8">
+        <f>IF(J67="","",G67*J67)</f>
+        <v/>
+      </c>
+      <c r="L67" s="8">
+        <f>IF(J67="",I67,K67)</f>
+        <v/>
+      </c>
+      <c r="M67" s="8">
+        <f>IF(J67="","",K67-I67)</f>
+        <v/>
+      </c>
+      <c r="N67" s="10" t="n"/>
+      <c r="O67" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P67" s="6" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n">
+        <v>56</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>Kaki karet</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr"/>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>Stabil &amp; anti gores</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="H68" s="8" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I68" s="8">
+        <f>G68*H68</f>
+        <v/>
+      </c>
+      <c r="J68" s="9" t="n"/>
+      <c r="K68" s="8">
+        <f>IF(J68="","",G68*J68)</f>
+        <v/>
+      </c>
+      <c r="L68" s="8">
+        <f>IF(J68="",I68,K68)</f>
+        <v/>
+      </c>
+      <c r="M68" s="8">
+        <f>IF(J68="","",K68-I68)</f>
+        <v/>
+      </c>
+      <c r="N68" s="10" t="n"/>
+      <c r="O68" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P68" s="6" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="n"/>
+      <c r="B69" s="12" t="inlineStr">
         <is>
           <t>Subtotal Mekanis — Struktur &amp; Panel — paket inti</t>
         </is>
       </c>
-      <c r="C67" s="12" t="n"/>
-      <c r="D67" s="12" t="n"/>
-      <c r="E67" s="12" t="n"/>
-      <c r="F67" s="12" t="n"/>
-      <c r="G67" s="12" t="n"/>
-      <c r="H67" s="12" t="n"/>
-      <c r="I67" s="13">
-        <f>SUMIFS(I59:I66,E59:E66,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J67" s="12" t="n"/>
-      <c r="K67" s="13">
-        <f>SUMIFS(K59:K66,E59:E66,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L67" s="13">
-        <f>SUMIFS(L59:L66,E59:E66,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M67" s="12" t="n"/>
-      <c r="N67" s="12" t="n"/>
-      <c r="O67" s="12" t="n"/>
-      <c r="P67" s="12" t="n"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
+      <c r="C69" s="12" t="n"/>
+      <c r="D69" s="12" t="n"/>
+      <c r="E69" s="12" t="n"/>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="n"/>
+      <c r="H69" s="12" t="n"/>
+      <c r="I69" s="13">
+        <f>SUMIFS(I61:I68,E61:E68,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J69" s="12" t="n"/>
+      <c r="K69" s="13">
+        <f>SUMIFS(K61:K68,E61:E68,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L69" s="13">
+        <f>SUMIFS(L61:L68,E61:E68,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M69" s="12" t="n"/>
+      <c r="N69" s="12" t="n"/>
+      <c r="O69" s="12" t="n"/>
+      <c r="P69" s="12" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>D. BAHAN HABIS PAKAI</t>
         </is>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="n">
-        <v>55</v>
-      </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>Lem PVC</t>
-        </is>
-      </c>
-      <c r="C70" s="6" t="inlineStr"/>
-      <c r="D70" s="6" t="inlineStr">
-        <is>
-          <t>Sambungan PVC</t>
-        </is>
-      </c>
-      <c r="E70" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F70" s="5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G70" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H70" s="8" t="n">
-        <v>15000</v>
-      </c>
-      <c r="I70" s="8">
-        <f>G70*H70</f>
-        <v/>
-      </c>
-      <c r="J70" s="9" t="n"/>
-      <c r="K70" s="8">
-        <f>IF(J70="","",G70*J70)</f>
-        <v/>
-      </c>
-      <c r="L70" s="8">
-        <f>IF(J70="",I70,K70)</f>
-        <v/>
-      </c>
-      <c r="M70" s="8">
-        <f>IF(J70="","",K70-I70)</f>
-        <v/>
-      </c>
-      <c r="N70" s="10" t="n"/>
-      <c r="O70" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P70" s="6" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="n">
-        <v>56</v>
-      </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>Lem akrilik (solvent)</t>
-        </is>
-      </c>
-      <c r="C71" s="6" t="inlineStr"/>
-      <c r="D71" s="6" t="inlineStr">
-        <is>
-          <t>Sambungan akrilik</t>
-        </is>
-      </c>
-      <c r="E71" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F71" s="5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G71" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H71" s="8" t="n">
-        <v>20000</v>
-      </c>
-      <c r="I71" s="8">
-        <f>G71*H71</f>
-        <v/>
-      </c>
-      <c r="J71" s="9" t="n"/>
-      <c r="K71" s="8">
-        <f>IF(J71="","",G71*J71)</f>
-        <v/>
-      </c>
-      <c r="L71" s="8">
-        <f>IF(J71="",I71,K71)</f>
-        <v/>
-      </c>
-      <c r="M71" s="8">
-        <f>IF(J71="","",K71-I71)</f>
-        <v/>
-      </c>
-      <c r="N71" s="10" t="n"/>
-      <c r="O71" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P71" s="6" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="n">
@@ -4258,17 +4268,13 @@
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>Sealant silikon akuarium</t>
-        </is>
-      </c>
-      <c r="C72" s="6" t="inlineStr">
-        <is>
-          <t>Tabung ± 300 mL</t>
-        </is>
-      </c>
+          <t>Lem PVC</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr"/>
       <c r="D72" s="6" t="inlineStr">
         <is>
-          <t>Kedap air sambungan &amp; bulkhead</t>
+          <t>Sambungan PVC</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -4285,7 +4291,7 @@
         <v>1</v>
       </c>
       <c r="H72" s="8" t="n">
-        <v>35000</v>
+        <v>15000</v>
       </c>
       <c r="I72" s="8">
         <f>G72*H72</f>
@@ -4318,13 +4324,13 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>Seal tape</t>
+          <t>Lem akrilik (solvent)</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr"/>
       <c r="D73" s="6" t="inlineStr">
         <is>
-          <t>Sambungan ulir</t>
+          <t>Sambungan akrilik</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -4334,14 +4340,14 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>roll</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G73" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H73" s="8" t="n">
-        <v>3000</v>
+        <v>20000</v>
       </c>
       <c r="I73" s="8">
         <f>G73*H73</f>
@@ -4374,17 +4380,17 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>Pewarna makanan</t>
+          <t>Sealant silikon akuarium</t>
         </is>
       </c>
       <c r="C74" s="6" t="inlineStr">
         <is>
-          <t>Warna gelap</t>
+          <t>Tabung ± 300 mL</t>
         </is>
       </c>
       <c r="D74" s="6" t="inlineStr">
         <is>
-          <t>Kontras kolom manometer</t>
+          <t>Kedap air sambungan &amp; bulkhead</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -4394,14 +4400,14 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>botol</t>
+          <t>pcs</t>
         </is>
       </c>
       <c r="G74" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H74" s="8" t="n">
-        <v>5000</v>
+        <v>35000</v>
       </c>
       <c r="I74" s="8">
         <f>G74*H74</f>
@@ -4426,11 +4432,7 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P74" s="6" t="inlineStr">
-        <is>
-          <t>Jangan disuntik untuk visual aliran (seluruh tangki ikut berwarna)</t>
-        </is>
-      </c>
+      <c r="P74" s="6" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="n">
@@ -4438,13 +4440,13 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>Amplas &amp; perlengkapan finishing</t>
+          <t>Seal tape</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr"/>
       <c r="D75" s="6" t="inlineStr">
         <is>
-          <t>Merapikan hasil cetak &amp; potongan</t>
+          <t>Sambungan ulir</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -4454,14 +4456,14 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>paket</t>
+          <t>roll</t>
         </is>
       </c>
       <c r="G75" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H75" s="8" t="n">
-        <v>15000</v>
+        <v>3000</v>
       </c>
       <c r="I75" s="8">
         <f>G75*H75</f>
@@ -4489,168 +4491,160 @@
       <c r="P75" s="6" t="inlineStr"/>
     </row>
     <row r="76">
-      <c r="A76" s="12" t="n"/>
-      <c r="B76" s="12" t="inlineStr">
+      <c r="A76" s="5" t="n">
+        <v>61</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>Pewarna makanan</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>Warna gelap</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>Kontras kolom manometer</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>botol</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H76" s="8" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I76" s="8">
+        <f>G76*H76</f>
+        <v/>
+      </c>
+      <c r="J76" s="9" t="n"/>
+      <c r="K76" s="8">
+        <f>IF(J76="","",G76*J76)</f>
+        <v/>
+      </c>
+      <c r="L76" s="8">
+        <f>IF(J76="",I76,K76)</f>
+        <v/>
+      </c>
+      <c r="M76" s="8">
+        <f>IF(J76="","",K76-I76)</f>
+        <v/>
+      </c>
+      <c r="N76" s="10" t="n"/>
+      <c r="O76" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P76" s="6" t="inlineStr">
+        <is>
+          <t>Jangan disuntik untuk visual aliran (seluruh tangki ikut berwarna)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n">
+        <v>62</v>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>Amplas &amp; perlengkapan finishing</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr"/>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>Merapikan hasil cetak &amp; potongan</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>paket</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H77" s="8" t="n">
+        <v>15000</v>
+      </c>
+      <c r="I77" s="8">
+        <f>G77*H77</f>
+        <v/>
+      </c>
+      <c r="J77" s="9" t="n"/>
+      <c r="K77" s="8">
+        <f>IF(J77="","",G77*J77)</f>
+        <v/>
+      </c>
+      <c r="L77" s="8">
+        <f>IF(J77="",I77,K77)</f>
+        <v/>
+      </c>
+      <c r="M77" s="8">
+        <f>IF(J77="","",K77-I77)</f>
+        <v/>
+      </c>
+      <c r="N77" s="10" t="n"/>
+      <c r="O77" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P77" s="6" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="12" t="n"/>
+      <c r="B78" s="12" t="inlineStr">
         <is>
           <t>Subtotal Bahan Habis Pakai — paket inti</t>
         </is>
       </c>
-      <c r="C76" s="12" t="n"/>
-      <c r="D76" s="12" t="n"/>
-      <c r="E76" s="12" t="n"/>
-      <c r="F76" s="12" t="n"/>
-      <c r="G76" s="12" t="n"/>
-      <c r="H76" s="12" t="n"/>
-      <c r="I76" s="13">
-        <f>SUMIFS(I70:I75,E70:E75,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J76" s="12" t="n"/>
-      <c r="K76" s="13">
-        <f>SUMIFS(K70:K75,E70:E75,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L76" s="13">
-        <f>SUMIFS(L70:L75,E70:E75,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M76" s="12" t="n"/>
-      <c r="N76" s="12" t="n"/>
-      <c r="O76" s="12" t="n"/>
-      <c r="P76" s="12" t="n"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
+      <c r="C78" s="12" t="n"/>
+      <c r="D78" s="12" t="n"/>
+      <c r="E78" s="12" t="n"/>
+      <c r="F78" s="12" t="n"/>
+      <c r="G78" s="12" t="n"/>
+      <c r="H78" s="12" t="n"/>
+      <c r="I78" s="13">
+        <f>SUMIFS(I72:I77,E72:E77,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J78" s="12" t="n"/>
+      <c r="K78" s="13">
+        <f>SUMIFS(K72:K77,E72:E77,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L78" s="13">
+        <f>SUMIFS(L72:L77,E72:E77,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M78" s="12" t="n"/>
+      <c r="N78" s="12" t="n"/>
+      <c r="O78" s="12" t="n"/>
+      <c r="P78" s="12" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>E. ALAT BANTU &amp; KALIBRASI (isi jumlah 0 jika sudah punya)</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="5" t="n">
-        <v>61</v>
-      </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>Jangka sorong digital</t>
-        </is>
-      </c>
-      <c r="C79" s="6" t="inlineStr">
-        <is>
-          <t>0–150 mm, resolusi 0,01 mm</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>Ukur ID pipa &amp; leher venturi</t>
-        </is>
-      </c>
-      <c r="E79" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F79" s="5" t="inlineStr">
-        <is>
-          <t>pcs</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H79" s="8" t="n">
-        <v>80000</v>
-      </c>
-      <c r="I79" s="8">
-        <f>G79*H79</f>
-        <v/>
-      </c>
-      <c r="J79" s="9" t="n"/>
-      <c r="K79" s="8">
-        <f>IF(J79="","",G79*J79)</f>
-        <v/>
-      </c>
-      <c r="L79" s="8">
-        <f>IF(J79="",I79,K79)</f>
-        <v/>
-      </c>
-      <c r="M79" s="8">
-        <f>IF(J79="","",K79-I79)</f>
-        <v/>
-      </c>
-      <c r="N79" s="10" t="n"/>
-      <c r="O79" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P79" s="6" t="inlineStr">
-        <is>
-          <t>Isi jumlah 0 kalau sudah punya</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="n">
-        <v>62</v>
-      </c>
-      <c r="B80" s="6" t="inlineStr">
-        <is>
-          <t>Mata bor 9,5 / 10 / 10,5 mm</t>
-        </is>
-      </c>
-      <c r="C80" s="6" t="inlineStr">
-        <is>
-          <t>Dipakai sebagai batang ukur</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>Cek diameter leher venturi</t>
-        </is>
-      </c>
-      <c r="E80" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F80" s="5" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H80" s="8" t="n">
-        <v>30000</v>
-      </c>
-      <c r="I80" s="8">
-        <f>G80*H80</f>
-        <v/>
-      </c>
-      <c r="J80" s="9" t="n"/>
-      <c r="K80" s="8">
-        <f>IF(J80="","",G80*J80)</f>
-        <v/>
-      </c>
-      <c r="L80" s="8">
-        <f>IF(J80="",I80,K80)</f>
-        <v/>
-      </c>
-      <c r="M80" s="8">
-        <f>IF(J80="","",K80-I80)</f>
-        <v/>
-      </c>
-      <c r="N80" s="10" t="n"/>
-      <c r="O80" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P80" s="6" t="inlineStr">
-        <is>
-          <t>Pengganti pin gauge yang mahal</t>
         </is>
       </c>
     </row>
@@ -4660,17 +4654,17 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>Gelas ukur 2 L</t>
+          <t>Jangka sorong digital</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
         <is>
-          <t>Skala 50 mL</t>
+          <t>0–150 mm, resolusi 0,01 mm</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>Kalibrasi volumetrik S1</t>
+          <t>Ukur ID pipa &amp; leher venturi</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -4687,7 +4681,7 @@
         <v>1</v>
       </c>
       <c r="H81" s="8" t="n">
-        <v>35000</v>
+        <v>80000</v>
       </c>
       <c r="I81" s="8">
         <f>G81*H81</f>
@@ -4714,7 +4708,7 @@
       </c>
       <c r="P81" s="6" t="inlineStr">
         <is>
-          <t>Stopwatch pakai HP</t>
+          <t>Isi jumlah 0 kalau sudah punya</t>
         </is>
       </c>
     </row>
@@ -4724,13 +4718,17 @@
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>Ember 15–20 L</t>
-        </is>
-      </c>
-      <c r="C82" s="6" t="inlineStr"/>
+          <t>Mata bor 9,5 / 10 / 10,5 mm</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>Dipakai sebagai batang ukur</t>
+        </is>
+      </c>
       <c r="D82" s="6" t="inlineStr">
         <is>
-          <t>Tangki sementara uji bangku</t>
+          <t>Cek diameter leher venturi</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -4740,14 +4738,14 @@
       </c>
       <c r="F82" s="5" t="inlineStr">
         <is>
-          <t>pcs</t>
+          <t>set</t>
         </is>
       </c>
       <c r="G82" s="7" t="n">
         <v>1</v>
       </c>
       <c r="H82" s="8" t="n">
-        <v>25000</v>
+        <v>30000</v>
       </c>
       <c r="I82" s="8">
         <f>G82*H82</f>
@@ -4772,7 +4770,11 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P82" s="6" t="inlineStr"/>
+      <c r="P82" s="6" t="inlineStr">
+        <is>
+          <t>Pengganti pin gauge yang mahal</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="5" t="n">
@@ -4780,13 +4782,17 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>Waterpass / selang air</t>
-        </is>
-      </c>
-      <c r="C83" s="6" t="inlineStr"/>
+          <t>Gelas ukur 2 L</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>Skala 50 mL</t>
+        </is>
+      </c>
       <c r="D83" s="6" t="inlineStr">
         <is>
-          <t>Sejajarkan datum &amp; angka 0 skala</t>
+          <t>Kalibrasi volumetrik S1</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -4803,7 +4809,7 @@
         <v>1</v>
       </c>
       <c r="H83" s="8" t="n">
-        <v>25000</v>
+        <v>35000</v>
       </c>
       <c r="I83" s="8">
         <f>G83*H83</f>
@@ -4828,311 +4834,315 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P83" s="6" t="inlineStr"/>
+      <c r="P83" s="6" t="inlineStr">
+        <is>
+          <t>Stopwatch pakai HP</t>
+        </is>
+      </c>
     </row>
     <row r="84">
-      <c r="A84" s="12" t="n"/>
-      <c r="B84" s="12" t="inlineStr">
+      <c r="A84" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>Ember 15–20 L</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr"/>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>Tangki sementara uji bangku</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G84" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" s="8" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I84" s="8">
+        <f>G84*H84</f>
+        <v/>
+      </c>
+      <c r="J84" s="9" t="n"/>
+      <c r="K84" s="8">
+        <f>IF(J84="","",G84*J84)</f>
+        <v/>
+      </c>
+      <c r="L84" s="8">
+        <f>IF(J84="",I84,K84)</f>
+        <v/>
+      </c>
+      <c r="M84" s="8">
+        <f>IF(J84="","",K84-I84)</f>
+        <v/>
+      </c>
+      <c r="N84" s="10" t="n"/>
+      <c r="O84" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P84" s="6" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="n">
+        <v>67</v>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>Waterpass / selang air</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr"/>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>Sejajarkan datum &amp; angka 0 skala</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="G85" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" s="8" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I85" s="8">
+        <f>G85*H85</f>
+        <v/>
+      </c>
+      <c r="J85" s="9" t="n"/>
+      <c r="K85" s="8">
+        <f>IF(J85="","",G85*J85)</f>
+        <v/>
+      </c>
+      <c r="L85" s="8">
+        <f>IF(J85="",I85,K85)</f>
+        <v/>
+      </c>
+      <c r="M85" s="8">
+        <f>IF(J85="","",K85-I85)</f>
+        <v/>
+      </c>
+      <c r="N85" s="10" t="n"/>
+      <c r="O85" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P85" s="6" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="12" t="n"/>
+      <c r="B86" s="12" t="inlineStr">
         <is>
           <t>Subtotal Alat Bantu &amp; Kalibrasi — paket inti</t>
         </is>
       </c>
-      <c r="C84" s="12" t="n"/>
-      <c r="D84" s="12" t="n"/>
-      <c r="E84" s="12" t="n"/>
-      <c r="F84" s="12" t="n"/>
-      <c r="G84" s="12" t="n"/>
-      <c r="H84" s="12" t="n"/>
-      <c r="I84" s="13">
-        <f>SUMIFS(I79:I83,E79:E83,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J84" s="12" t="n"/>
-      <c r="K84" s="13">
-        <f>SUMIFS(K79:K83,E79:E83,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L84" s="13">
-        <f>SUMIFS(L79:L83,E79:E83,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M84" s="12" t="n"/>
-      <c r="N84" s="12" t="n"/>
-      <c r="O84" s="12" t="n"/>
-      <c r="P84" s="12" t="n"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="4" t="inlineStr">
+      <c r="C86" s="12" t="n"/>
+      <c r="D86" s="12" t="n"/>
+      <c r="E86" s="12" t="n"/>
+      <c r="F86" s="12" t="n"/>
+      <c r="G86" s="12" t="n"/>
+      <c r="H86" s="12" t="n"/>
+      <c r="I86" s="13">
+        <f>SUMIFS(I81:I85,E81:E85,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J86" s="12" t="n"/>
+      <c r="K86" s="13">
+        <f>SUMIFS(K81:K85,E81:E85,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L86" s="13">
+        <f>SUMIFS(L81:L85,E81:E85,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M86" s="12" t="n"/>
+      <c r="N86" s="12" t="n"/>
+      <c r="O86" s="12" t="n"/>
+      <c r="P86" s="12" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>F. BIAYA LAIN</t>
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="5" t="n">
-        <v>66</v>
-      </c>
-      <c r="B87" s="6" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="5" t="n">
+        <v>68</v>
+      </c>
+      <c r="B89" s="6" t="inlineStr">
         <is>
           <t>Ongkos kirim</t>
         </is>
       </c>
-      <c r="C87" s="6" t="inlineStr">
+      <c r="C89" s="6" t="inlineStr">
         <is>
           <t>Perkiraan beberapa toko</t>
         </is>
       </c>
-      <c r="D87" s="6" t="inlineStr"/>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F87" s="5" t="inlineStr">
+      <c r="D89" s="6" t="inlineStr"/>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
         <is>
           <t>paket</t>
         </is>
       </c>
-      <c r="G87" s="7" t="n">
+      <c r="G89" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H87" s="8" t="n">
+      <c r="H89" s="8" t="n">
         <v>100000</v>
       </c>
-      <c r="I87" s="8">
-        <f>G87*H87</f>
-        <v/>
-      </c>
-      <c r="J87" s="9" t="n"/>
-      <c r="K87" s="8">
-        <f>IF(J87="","",G87*J87)</f>
-        <v/>
-      </c>
-      <c r="L87" s="8">
-        <f>IF(J87="",I87,K87)</f>
-        <v/>
-      </c>
-      <c r="M87" s="8">
-        <f>IF(J87="","",K87-I87)</f>
-        <v/>
-      </c>
-      <c r="N87" s="10" t="n"/>
-      <c r="O87" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P87" s="6" t="inlineStr">
+      <c r="I89" s="8">
+        <f>G89*H89</f>
+        <v/>
+      </c>
+      <c r="J89" s="9" t="n"/>
+      <c r="K89" s="8">
+        <f>IF(J89="","",G89*J89)</f>
+        <v/>
+      </c>
+      <c r="L89" s="8">
+        <f>IF(J89="",I89,K89)</f>
+        <v/>
+      </c>
+      <c r="M89" s="8">
+        <f>IF(J89="","",K89-I89)</f>
+        <v/>
+      </c>
+      <c r="N89" s="10" t="n"/>
+      <c r="O89" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P89" s="6" t="inlineStr">
         <is>
           <t>Sesuaikan setelah checkout</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="5" t="n">
-        <v>67</v>
-      </c>
-      <c r="B88" s="6" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="5" t="n">
+        <v>69</v>
+      </c>
+      <c r="B90" s="6" t="inlineStr">
         <is>
           <t>Transport belanja lokal</t>
         </is>
       </c>
-      <c r="C88" s="6" t="inlineStr">
+      <c r="C90" s="6" t="inlineStr">
         <is>
           <t>Toko bangunan, akrilik, elektronik</t>
         </is>
       </c>
-      <c r="D88" s="6" t="inlineStr"/>
-      <c r="E88" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F88" s="5" t="inlineStr">
+      <c r="D90" s="6" t="inlineStr"/>
+      <c r="E90" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
         <is>
           <t>paket</t>
         </is>
       </c>
-      <c r="G88" s="7" t="n">
+      <c r="G90" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="H88" s="8" t="n">
+      <c r="H90" s="8" t="n">
         <v>50000</v>
       </c>
-      <c r="I88" s="8">
-        <f>G88*H88</f>
-        <v/>
-      </c>
-      <c r="J88" s="9" t="n"/>
-      <c r="K88" s="8">
-        <f>IF(J88="","",G88*J88)</f>
-        <v/>
-      </c>
-      <c r="L88" s="8">
-        <f>IF(J88="",I88,K88)</f>
-        <v/>
-      </c>
-      <c r="M88" s="8">
-        <f>IF(J88="","",K88-I88)</f>
-        <v/>
-      </c>
-      <c r="N88" s="10" t="n"/>
-      <c r="O88" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P88" s="6" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="12" t="n"/>
-      <c r="B89" s="12" t="inlineStr">
+      <c r="I90" s="8">
+        <f>G90*H90</f>
+        <v/>
+      </c>
+      <c r="J90" s="9" t="n"/>
+      <c r="K90" s="8">
+        <f>IF(J90="","",G90*J90)</f>
+        <v/>
+      </c>
+      <c r="L90" s="8">
+        <f>IF(J90="",I90,K90)</f>
+        <v/>
+      </c>
+      <c r="M90" s="8">
+        <f>IF(J90="","",K90-I90)</f>
+        <v/>
+      </c>
+      <c r="N90" s="10" t="n"/>
+      <c r="O90" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P90" s="6" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="n"/>
+      <c r="B91" s="12" t="inlineStr">
         <is>
           <t>Subtotal Biaya Lain — paket inti</t>
         </is>
       </c>
-      <c r="C89" s="12" t="n"/>
-      <c r="D89" s="12" t="n"/>
-      <c r="E89" s="12" t="n"/>
-      <c r="F89" s="12" t="n"/>
-      <c r="G89" s="12" t="n"/>
-      <c r="H89" s="12" t="n"/>
-      <c r="I89" s="13">
-        <f>SUMIFS(I87:I88,E87:E88,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J89" s="12" t="n"/>
-      <c r="K89" s="13">
-        <f>SUMIFS(K87:K88,E87:E88,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L89" s="13">
-        <f>SUMIFS(L87:L88,E87:E88,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M89" s="12" t="n"/>
-      <c r="N89" s="12" t="n"/>
-      <c r="O89" s="12" t="n"/>
-      <c r="P89" s="12" t="n"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="4" t="inlineStr">
+      <c r="C91" s="12" t="n"/>
+      <c r="D91" s="12" t="n"/>
+      <c r="E91" s="12" t="n"/>
+      <c r="F91" s="12" t="n"/>
+      <c r="G91" s="12" t="n"/>
+      <c r="H91" s="12" t="n"/>
+      <c r="I91" s="13">
+        <f>SUMIFS(I89:I90,E89:E90,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J91" s="12" t="n"/>
+      <c r="K91" s="13">
+        <f>SUMIFS(K89:K90,E89:E90,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L91" s="13">
+        <f>SUMIFS(L89:L90,E89:E90,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M91" s="12" t="n"/>
+      <c r="N91" s="12" t="n"/>
+      <c r="O91" s="12" t="n"/>
+      <c r="P91" s="12" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
         <is>
           <t>G. JASA</t>
         </is>
       </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="5" t="n">
-        <v>68</v>
-      </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>Desain &amp; perhitungan</t>
-        </is>
-      </c>
-      <c r="C92" s="6" t="inlineStr">
-        <is>
-          <t>Rev. 01–08, profil manometer, sketsa</t>
-        </is>
-      </c>
-      <c r="D92" s="6" t="inlineStr"/>
-      <c r="E92" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F92" s="5" t="inlineStr">
-        <is>
-          <t>paket</t>
-        </is>
-      </c>
-      <c r="G92" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H92" s="8" t="n">
-        <v>250000</v>
-      </c>
-      <c r="I92" s="8">
-        <f>G92*H92</f>
-        <v/>
-      </c>
-      <c r="J92" s="14" t="n"/>
-      <c r="K92" s="8">
-        <f>IF(J92="","",G92*J92)</f>
-        <v/>
-      </c>
-      <c r="L92" s="8">
-        <f>IF(J92="",I92,K92)</f>
-        <v/>
-      </c>
-      <c r="M92" s="8">
-        <f>IF(J92="","",K92-I92)</f>
-        <v/>
-      </c>
-      <c r="N92" s="15" t="n"/>
-      <c r="O92" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P92" s="6" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="5" t="n">
-        <v>69</v>
-      </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>Uji bangku &amp; penyesuaian</t>
-        </is>
-      </c>
-      <c r="C93" s="6" t="inlineStr">
-        <is>
-          <t>Pompa, S1, katup searah, venturi</t>
-        </is>
-      </c>
-      <c r="D93" s="6" t="inlineStr"/>
-      <c r="E93" s="5" t="inlineStr">
-        <is>
-          <t>Inti</t>
-        </is>
-      </c>
-      <c r="F93" s="5" t="inlineStr">
-        <is>
-          <t>paket</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H93" s="8" t="n">
-        <v>150000</v>
-      </c>
-      <c r="I93" s="8">
-        <f>G93*H93</f>
-        <v/>
-      </c>
-      <c r="J93" s="14" t="n"/>
-      <c r="K93" s="8">
-        <f>IF(J93="","",G93*J93)</f>
-        <v/>
-      </c>
-      <c r="L93" s="8">
-        <f>IF(J93="",I93,K93)</f>
-        <v/>
-      </c>
-      <c r="M93" s="8">
-        <f>IF(J93="","",K93-I93)</f>
-        <v/>
-      </c>
-      <c r="N93" s="15" t="n"/>
-      <c r="O93" s="7" t="inlineStr">
-        <is>
-          <t>Belum</t>
-        </is>
-      </c>
-      <c r="P93" s="6" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="5" t="n">
@@ -5140,12 +5150,12 @@
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>Perakitan mekanik &amp; hidrolik</t>
+          <t>Desain &amp; perhitungan</t>
         </is>
       </c>
       <c r="C94" s="6" t="inlineStr">
         <is>
-          <t>Pipa, venturi, panel manometer, uji bocor 24 jam</t>
+          <t>Rev. 01–08, profil manometer, sketsa</t>
         </is>
       </c>
       <c r="D94" s="6" t="inlineStr"/>
@@ -5163,7 +5173,7 @@
         <v>1</v>
       </c>
       <c r="H94" s="8" t="n">
-        <v>400000</v>
+        <v>250000</v>
       </c>
       <c r="I94" s="8">
         <f>G94*H94</f>
@@ -5196,12 +5206,12 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>Elektronik &amp; firmware</t>
+          <t>Uji bangku &amp; penyesuaian</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>Kontrol PI, ukur periode pulsa, pengaman luapan, LCD, tombol CEK, log serial</t>
+          <t>Pompa, S1, katup searah, venturi</t>
         </is>
       </c>
       <c r="D95" s="6" t="inlineStr"/>
@@ -5219,7 +5229,7 @@
         <v>1</v>
       </c>
       <c r="H95" s="8" t="n">
-        <v>450000</v>
+        <v>150000</v>
       </c>
       <c r="I95" s="8">
         <f>G95*H95</f>
@@ -5252,12 +5262,12 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>Kalibrasi &amp; laporan kalibrasi</t>
+          <t>Perakitan mekanik &amp; hidrolik</t>
         </is>
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>Kalibrasi volumetrik S1, uji nol, ukur leher venturi</t>
+          <t>Pipa, venturi, panel manometer, uji bocor 24 jam</t>
         </is>
       </c>
       <c r="D96" s="6" t="inlineStr"/>
@@ -5275,7 +5285,7 @@
         <v>1</v>
       </c>
       <c r="H96" s="8" t="n">
-        <v>150000</v>
+        <v>400000</v>
       </c>
       <c r="I96" s="8">
         <f>G96*H96</f>
@@ -5308,12 +5318,12 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>Dokumentasi</t>
+          <t>Elektronik &amp; firmware</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>SOP, manual alat, diagram rangkaian</t>
+          <t>Kontrol PI, ukur periode pulsa, pengaman luapan, LCD, tombol CEK, log serial</t>
         </is>
       </c>
       <c r="D97" s="6" t="inlineStr"/>
@@ -5331,7 +5341,7 @@
         <v>1</v>
       </c>
       <c r="H97" s="8" t="n">
-        <v>100000</v>
+        <v>450000</v>
       </c>
       <c r="I97" s="8">
         <f>G97*H97</f>
@@ -5356,30 +5366,26 @@
           <t>Belum</t>
         </is>
       </c>
-      <c r="P97" s="6" t="inlineStr">
-        <is>
-          <t>Bukan LKPD/instrumen penelitian (itu isi skripsi client)</t>
-        </is>
-      </c>
+      <c r="P97" s="6" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="5" t="n">
         <v>74</v>
       </c>
-      <c r="B98" s="11" t="inlineStr">
-        <is>
-          <t>Jasa tambahan paket lengkap</t>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>Kalibrasi &amp; laporan kalibrasi</t>
         </is>
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Zona C + S2 + uji rugi tekanan S2</t>
+          <t>Kalibrasi volumetrik S1, uji nol, ukur leher venturi</t>
         </is>
       </c>
       <c r="D98" s="6" t="inlineStr"/>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>Lengkap</t>
+          <t>Inti</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
@@ -5391,7 +5397,7 @@
         <v>1</v>
       </c>
       <c r="H98" s="8" t="n">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I98" s="8">
         <f>G98*H98</f>
@@ -5419,52 +5425,168 @@
       <c r="P98" s="6" t="inlineStr"/>
     </row>
     <row r="99">
-      <c r="A99" s="12" t="n"/>
-      <c r="B99" s="12" t="inlineStr">
+      <c r="A99" s="5" t="n">
+        <v>75</v>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>Dokumentasi</t>
+        </is>
+      </c>
+      <c r="C99" s="6" t="inlineStr">
+        <is>
+          <t>SOP, manual alat, diagram rangkaian</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr"/>
+      <c r="E99" s="5" t="inlineStr">
+        <is>
+          <t>Inti</t>
+        </is>
+      </c>
+      <c r="F99" s="5" t="inlineStr">
+        <is>
+          <t>paket</t>
+        </is>
+      </c>
+      <c r="G99" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H99" s="8" t="n">
+        <v>100000</v>
+      </c>
+      <c r="I99" s="8">
+        <f>G99*H99</f>
+        <v/>
+      </c>
+      <c r="J99" s="14" t="n"/>
+      <c r="K99" s="8">
+        <f>IF(J99="","",G99*J99)</f>
+        <v/>
+      </c>
+      <c r="L99" s="8">
+        <f>IF(J99="",I99,K99)</f>
+        <v/>
+      </c>
+      <c r="M99" s="8">
+        <f>IF(J99="","",K99-I99)</f>
+        <v/>
+      </c>
+      <c r="N99" s="15" t="n"/>
+      <c r="O99" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P99" s="6" t="inlineStr">
+        <is>
+          <t>Bukan LKPD/instrumen penelitian (itu isi skripsi client)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>Jasa tambahan paket lengkap</t>
+        </is>
+      </c>
+      <c r="C100" s="6" t="inlineStr">
+        <is>
+          <t>Zona C + S2 + uji rugi tekanan S2</t>
+        </is>
+      </c>
+      <c r="D100" s="6" t="inlineStr"/>
+      <c r="E100" s="5" t="inlineStr">
+        <is>
+          <t>Lengkap</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>paket</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H100" s="8" t="n">
+        <v>200000</v>
+      </c>
+      <c r="I100" s="8">
+        <f>G100*H100</f>
+        <v/>
+      </c>
+      <c r="J100" s="14" t="n"/>
+      <c r="K100" s="8">
+        <f>IF(J100="","",G100*J100)</f>
+        <v/>
+      </c>
+      <c r="L100" s="8">
+        <f>IF(J100="",I100,K100)</f>
+        <v/>
+      </c>
+      <c r="M100" s="8">
+        <f>IF(J100="","",K100-I100)</f>
+        <v/>
+      </c>
+      <c r="N100" s="15" t="n"/>
+      <c r="O100" s="7" t="inlineStr">
+        <is>
+          <t>Belum</t>
+        </is>
+      </c>
+      <c r="P100" s="6" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="12" t="n"/>
+      <c r="B101" s="12" t="inlineStr">
         <is>
           <t>Subtotal Jasa — paket inti</t>
         </is>
       </c>
-      <c r="C99" s="12" t="n"/>
-      <c r="D99" s="12" t="n"/>
-      <c r="E99" s="12" t="n"/>
-      <c r="F99" s="12" t="n"/>
-      <c r="G99" s="12" t="n"/>
-      <c r="H99" s="12" t="n"/>
-      <c r="I99" s="13">
-        <f>SUMIFS(I92:I98,E92:E98,"Inti")</f>
-        <v/>
-      </c>
-      <c r="J99" s="12" t="n"/>
-      <c r="K99" s="13">
-        <f>SUMIFS(K92:K98,E92:E98,"Inti")</f>
-        <v/>
-      </c>
-      <c r="L99" s="13">
-        <f>SUMIFS(L92:L98,E92:E98,"Inti")</f>
-        <v/>
-      </c>
-      <c r="M99" s="12" t="n"/>
-      <c r="N99" s="12" t="n"/>
-      <c r="O99" s="12" t="n"/>
-      <c r="P99" s="12" t="n"/>
+      <c r="C101" s="12" t="n"/>
+      <c r="D101" s="12" t="n"/>
+      <c r="E101" s="12" t="n"/>
+      <c r="F101" s="12" t="n"/>
+      <c r="G101" s="12" t="n"/>
+      <c r="H101" s="12" t="n"/>
+      <c r="I101" s="13">
+        <f>SUMIFS(I94:I100,E94:E100,"Inti")</f>
+        <v/>
+      </c>
+      <c r="J101" s="12" t="n"/>
+      <c r="K101" s="13">
+        <f>SUMIFS(K94:K100,E94:E100,"Inti")</f>
+        <v/>
+      </c>
+      <c r="L101" s="13">
+        <f>SUMIFS(L94:L100,E94:E100,"Inti")</f>
+        <v/>
+      </c>
+      <c r="M101" s="12" t="n"/>
+      <c r="N101" s="12" t="n"/>
+      <c r="O101" s="12" t="n"/>
+      <c r="P101" s="12" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:P100"/>
+  <autoFilter ref="A5:P102"/>
   <mergeCells count="7">
-    <mergeCell ref="A31:P31"/>
+    <mergeCell ref="A60:P60"/>
+    <mergeCell ref="A93:P93"/>
+    <mergeCell ref="A80:P80"/>
+    <mergeCell ref="A88:P88"/>
     <mergeCell ref="A6:P6"/>
-    <mergeCell ref="A58:P58"/>
-    <mergeCell ref="A69:P69"/>
-    <mergeCell ref="A91:P91"/>
-    <mergeCell ref="A78:P78"/>
-    <mergeCell ref="A86:P86"/>
+    <mergeCell ref="A33:P33"/>
+    <mergeCell ref="A71:P71"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation sqref="E6:E100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E6:E102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Inti,Lengkap,Opsional"</formula1>
     </dataValidation>
-    <dataValidation sqref="O6:O100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O6:O102" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Belum,Dipesan,Diterima,Batal"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5582,19 +5704,19 @@
         </is>
       </c>
       <c r="B9" s="22">
-        <f>SUMIFS(RAB!$I$7:$I$28,RAB!$E$7:$E$28,"Inti")</f>
+        <f>SUMIFS(RAB!$I$7:$I$30,RAB!$E$7:$E$30,"Inti")</f>
         <v/>
       </c>
       <c r="C9" s="22">
-        <f>SUMIFS(RAB!$K$7:$K$28,RAB!$E$7:$E$28,"Inti")</f>
+        <f>SUMIFS(RAB!$K$7:$K$30,RAB!$E$7:$E$30,"Inti")</f>
         <v/>
       </c>
       <c r="D9" s="22">
-        <f>SUMIFS(RAB!$L$7:$L$28,RAB!$E$7:$E$28,"Inti")</f>
+        <f>SUMIFS(RAB!$L$7:$L$30,RAB!$E$7:$E$30,"Inti")</f>
         <v/>
       </c>
       <c r="E9" s="21">
-        <f>COUNTIFS(RAB!$E$7:$E$28,"Inti",RAB!$J$7:$J$28,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$7:$E$28,"Inti")</f>
+        <f>COUNTIFS(RAB!$E$7:$E$30,"Inti",RAB!$J$7:$J$30,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$7:$E$30,"Inti")</f>
         <v/>
       </c>
     </row>
@@ -5605,19 +5727,19 @@
         </is>
       </c>
       <c r="B10" s="22">
-        <f>SUMIFS(RAB!$I$32:$I$55,RAB!$E$32:$E$55,"Inti")</f>
+        <f>SUMIFS(RAB!$I$34:$I$57,RAB!$E$34:$E$57,"Inti")</f>
         <v/>
       </c>
       <c r="C10" s="22">
-        <f>SUMIFS(RAB!$K$32:$K$55,RAB!$E$32:$E$55,"Inti")</f>
+        <f>SUMIFS(RAB!$K$34:$K$57,RAB!$E$34:$E$57,"Inti")</f>
         <v/>
       </c>
       <c r="D10" s="22">
-        <f>SUMIFS(RAB!$L$32:$L$55,RAB!$E$32:$E$55,"Inti")</f>
+        <f>SUMIFS(RAB!$L$34:$L$57,RAB!$E$34:$E$57,"Inti")</f>
         <v/>
       </c>
       <c r="E10" s="21">
-        <f>COUNTIFS(RAB!$E$32:$E$55,"Inti",RAB!$J$32:$J$55,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$32:$E$55,"Inti")</f>
+        <f>COUNTIFS(RAB!$E$34:$E$57,"Inti",RAB!$J$34:$J$57,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$34:$E$57,"Inti")</f>
         <v/>
       </c>
     </row>
@@ -5628,19 +5750,19 @@
         </is>
       </c>
       <c r="B11" s="22">
-        <f>SUMIFS(RAB!$I$59:$I$66,RAB!$E$59:$E$66,"Inti")</f>
+        <f>SUMIFS(RAB!$I$61:$I$68,RAB!$E$61:$E$68,"Inti")</f>
         <v/>
       </c>
       <c r="C11" s="22">
-        <f>SUMIFS(RAB!$K$59:$K$66,RAB!$E$59:$E$66,"Inti")</f>
+        <f>SUMIFS(RAB!$K$61:$K$68,RAB!$E$61:$E$68,"Inti")</f>
         <v/>
       </c>
       <c r="D11" s="22">
-        <f>SUMIFS(RAB!$L$59:$L$66,RAB!$E$59:$E$66,"Inti")</f>
+        <f>SUMIFS(RAB!$L$61:$L$68,RAB!$E$61:$E$68,"Inti")</f>
         <v/>
       </c>
       <c r="E11" s="21">
-        <f>COUNTIFS(RAB!$E$59:$E$66,"Inti",RAB!$J$59:$J$66,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$59:$E$66,"Inti")</f>
+        <f>COUNTIFS(RAB!$E$61:$E$68,"Inti",RAB!$J$61:$J$68,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$61:$E$68,"Inti")</f>
         <v/>
       </c>
     </row>
@@ -5651,19 +5773,19 @@
         </is>
       </c>
       <c r="B12" s="22">
-        <f>SUMIFS(RAB!$I$70:$I$75,RAB!$E$70:$E$75,"Inti")</f>
+        <f>SUMIFS(RAB!$I$72:$I$77,RAB!$E$72:$E$77,"Inti")</f>
         <v/>
       </c>
       <c r="C12" s="22">
-        <f>SUMIFS(RAB!$K$70:$K$75,RAB!$E$70:$E$75,"Inti")</f>
+        <f>SUMIFS(RAB!$K$72:$K$77,RAB!$E$72:$E$77,"Inti")</f>
         <v/>
       </c>
       <c r="D12" s="22">
-        <f>SUMIFS(RAB!$L$70:$L$75,RAB!$E$70:$E$75,"Inti")</f>
+        <f>SUMIFS(RAB!$L$72:$L$77,RAB!$E$72:$E$77,"Inti")</f>
         <v/>
       </c>
       <c r="E12" s="21">
-        <f>COUNTIFS(RAB!$E$70:$E$75,"Inti",RAB!$J$70:$J$75,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$70:$E$75,"Inti")</f>
+        <f>COUNTIFS(RAB!$E$72:$E$77,"Inti",RAB!$J$72:$J$77,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$72:$E$77,"Inti")</f>
         <v/>
       </c>
     </row>
@@ -5674,19 +5796,19 @@
         </is>
       </c>
       <c r="B13" s="22">
-        <f>SUMIFS(RAB!$I$79:$I$83,RAB!$E$79:$E$83,"Inti")</f>
+        <f>SUMIFS(RAB!$I$81:$I$85,RAB!$E$81:$E$85,"Inti")</f>
         <v/>
       </c>
       <c r="C13" s="22">
-        <f>SUMIFS(RAB!$K$79:$K$83,RAB!$E$79:$E$83,"Inti")</f>
+        <f>SUMIFS(RAB!$K$81:$K$85,RAB!$E$81:$E$85,"Inti")</f>
         <v/>
       </c>
       <c r="D13" s="22">
-        <f>SUMIFS(RAB!$L$79:$L$83,RAB!$E$79:$E$83,"Inti")</f>
+        <f>SUMIFS(RAB!$L$81:$L$85,RAB!$E$81:$E$85,"Inti")</f>
         <v/>
       </c>
       <c r="E13" s="21">
-        <f>COUNTIFS(RAB!$E$79:$E$83,"Inti",RAB!$J$79:$J$83,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$79:$E$83,"Inti")</f>
+        <f>COUNTIFS(RAB!$E$81:$E$85,"Inti",RAB!$J$81:$J$85,"&lt;&gt;")&amp;" / "&amp;COUNTIFS(RAB!$E$81:$E$85,"Inti")</f>
         <v/>
       </c>
     </row>
@@ -5738,15 +5860,15 @@
         </is>
       </c>
       <c r="B16" s="22">
-        <f>SUMIFS(RAB!$I$87:$I$88,RAB!$E$87:$E$88,"Inti")</f>
+        <f>SUMIFS(RAB!$I$89:$I$90,RAB!$E$89:$E$90,"Inti")</f>
         <v/>
       </c>
       <c r="C16" s="22">
-        <f>SUMIFS(RAB!$K$87:$K$88,RAB!$E$87:$E$88,"Inti")</f>
+        <f>SUMIFS(RAB!$K$89:$K$90,RAB!$E$89:$E$90,"Inti")</f>
         <v/>
       </c>
       <c r="D16" s="22">
-        <f>SUMIFS(RAB!$L$87:$L$88,RAB!$E$87:$E$88,"Inti")</f>
+        <f>SUMIFS(RAB!$L$89:$L$90,RAB!$E$89:$E$90,"Inti")</f>
         <v/>
       </c>
       <c r="E16" s="21" t="inlineStr"/>
@@ -5775,12 +5897,12 @@
         </is>
       </c>
       <c r="B18" s="22">
-        <f>SUMIFS(RAB!$I$92:$I$98,RAB!$E$92:$E$98,"Inti")</f>
+        <f>SUMIFS(RAB!$I$94:$I$100,RAB!$E$94:$E$100,"Inti")</f>
         <v/>
       </c>
       <c r="C18" s="22" t="inlineStr"/>
       <c r="D18" s="22">
-        <f>SUMIFS(RAB!$L$92:$L$98,RAB!$E$92:$E$98,"Inti")</f>
+        <f>SUMIFS(RAB!$L$94:$L$100,RAB!$E$94:$E$100,"Inti")</f>
         <v/>
       </c>
       <c r="E18" s="21" t="inlineStr"/>
@@ -5905,15 +6027,15 @@
         </is>
       </c>
       <c r="B26" s="22">
-        <f>SUMIFS(RAB!$I$6:$I$100,RAB!$E$6:$E$100,"Lengkap")+(SUMIFS(RAB!$I$6:$I$100,RAB!$E$6:$E$100,"Lengkap")-SUMIFS(RAB!$I$92:$I$98,RAB!$E$92:$E$98,"Lengkap"))*$B$5</f>
+        <f>SUMIFS(RAB!$I$6:$I$102,RAB!$E$6:$E$102,"Lengkap")+(SUMIFS(RAB!$I$6:$I$102,RAB!$E$6:$E$102,"Lengkap")-SUMIFS(RAB!$I$94:$I$100,RAB!$E$94:$E$100,"Lengkap"))*$B$5</f>
         <v/>
       </c>
       <c r="C26" s="22">
-        <f>SUMIFS(RAB!$K$6:$K$100,RAB!$E$6:$E$100,"Lengkap")</f>
+        <f>SUMIFS(RAB!$K$6:$K$102,RAB!$E$6:$E$102,"Lengkap")</f>
         <v/>
       </c>
       <c r="D26" s="22">
-        <f>SUMIFS(RAB!$L$6:$L$100,RAB!$E$6:$E$100,"Lengkap")+(SUMIFS(RAB!$L$6:$L$100,RAB!$E$6:$E$100,"Lengkap")-SUMIFS(RAB!$L$92:$L$98,RAB!$E$92:$E$98,"Lengkap"))*$B$5</f>
+        <f>SUMIFS(RAB!$L$6:$L$102,RAB!$E$6:$E$102,"Lengkap")+(SUMIFS(RAB!$L$6:$L$102,RAB!$E$6:$E$102,"Lengkap")-SUMIFS(RAB!$L$94:$L$100,RAB!$E$94:$E$100,"Lengkap"))*$B$5</f>
         <v/>
       </c>
       <c r="E26" s="21" t="inlineStr">
@@ -5950,15 +6072,15 @@
         </is>
       </c>
       <c r="B28" s="22">
-        <f>SUMIFS(RAB!$I$6:$I$100,RAB!$E$6:$E$100,"Opsional")</f>
+        <f>SUMIFS(RAB!$I$6:$I$102,RAB!$E$6:$E$102,"Opsional")</f>
         <v/>
       </c>
       <c r="C28" s="22">
-        <f>SUMIFS(RAB!$K$6:$K$100,RAB!$E$6:$E$100,"Opsional")</f>
+        <f>SUMIFS(RAB!$K$6:$K$102,RAB!$E$6:$E$102,"Opsional")</f>
         <v/>
       </c>
       <c r="D28" s="22">
-        <f>SUMIFS(RAB!$L$6:$L$100,RAB!$E$6:$E$100,"Opsional")</f>
+        <f>SUMIFS(RAB!$L$6:$L$102,RAB!$E$6:$E$102,"Opsional")</f>
         <v/>
       </c>
       <c r="E28" s="21" t="inlineStr">

</xml_diff>

<commit_message>
Tambah jadwal harian, sheet keuangan, folder nota, dan harga beli sensor
</commit_message>
<xml_diff>
--- a/anggaran/RAB-alat-praktikum-rev08.xlsx
+++ b/anggaran/RAB-alat-praktikum-rev08.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAB" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keuangan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ringkasan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RAB'!$A$5:$P$102</definedName>
@@ -21,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="&quot;Rp&quot;#,##0;[Red]-&quot;Rp&quot;#,##0;&quot;-&quot;"/>
+    <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,6 +63,14 @@
       <b val="1"/>
       <color rgb="001F3A5F"/>
       <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="8">
@@ -127,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -212,6 +222,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -879,7 +902,9 @@
         <f>G9*H9</f>
         <v/>
       </c>
-      <c r="J9" s="9" t="n"/>
+      <c r="J9" s="9" t="n">
+        <v>29189</v>
+      </c>
       <c r="K9" s="8">
         <f>IF(J9="","",G9*J9)</f>
         <v/>
@@ -895,7 +920,7 @@
       <c r="N9" s="10" t="n"/>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Diterima</t>
         </is>
       </c>
       <c r="P9" s="6" t="inlineStr">
@@ -1993,7 +2018,9 @@
         <f>G27*H27</f>
         <v/>
       </c>
-      <c r="J27" s="9" t="n"/>
+      <c r="J27" s="9" t="n">
+        <v>42211</v>
+      </c>
       <c r="K27" s="8">
         <f>IF(J27="","",G27*J27)</f>
         <v/>
@@ -2009,7 +2036,7 @@
       <c r="N27" s="10" t="n"/>
       <c r="O27" s="7" t="inlineStr">
         <is>
-          <t>Belum</t>
+          <t>Diterima</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
@@ -2237,6 +2264,7 @@
       <c r="O31" s="12" t="n"/>
       <c r="P31" s="12" t="n"/>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
@@ -3741,6 +3769,7 @@
       <c r="O58" s="12" t="n"/>
       <c r="P58" s="12" t="n"/>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
@@ -4255,6 +4284,7 @@
       <c r="O69" s="12" t="n"/>
       <c r="P69" s="12" t="n"/>
     </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
@@ -4641,6 +4671,7 @@
       <c r="O78" s="12" t="n"/>
       <c r="P78" s="12" t="n"/>
     </row>
+    <row r="79"/>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
@@ -4983,6 +5014,7 @@
       <c r="O86" s="12" t="n"/>
       <c r="P86" s="12" t="n"/>
     </row>
+    <row r="87"/>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
@@ -5137,6 +5169,7 @@
       <c r="O91" s="12" t="n"/>
       <c r="P91" s="12" t="n"/>
     </row>
+    <row r="92"/>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
@@ -5599,6 +5632,1037 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:I62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>KEUANGAN PROYEK — dana masuk, pengeluaran, sisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sel kuning diisi. Simpan foto nota di folder anggaran/nota/ lalu tulis nama filenya di kolom File nota; kolom Link otomatis membukanya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="32" t="inlineStr">
+        <is>
+          <t>Buka folder nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>RINGKASAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>Dana diterima</t>
+        </is>
+      </c>
+      <c r="B6" s="35" t="n"/>
+      <c r="C6" s="35" t="n"/>
+      <c r="D6" s="13">
+        <f>D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="34" t="inlineStr">
+        <is>
+          <t>Sudah dipakai</t>
+        </is>
+      </c>
+      <c r="B7" s="35" t="n"/>
+      <c r="C7" s="35" t="n"/>
+      <c r="D7" s="13">
+        <f>E62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>Sisa dana</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="n"/>
+      <c r="C8" s="37" t="n"/>
+      <c r="D8" s="38">
+        <f>D6-D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="39">
+        <f>IF(D8&lt;0,"Dana kurang — minta tambahan","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>1. DANA MASUK</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Tanggal</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Jumlah</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>File nota / bukti</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="40" t="n"/>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>DP dari client</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="9" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="6">
+        <f>IF(G12="","",HYPERLINK("nota/"&amp;G12,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>Isi tanggal transfer</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="40" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="9" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="10" t="n"/>
+      <c r="H13" s="6">
+        <f>IF(G13="","",HYPERLINK("nota/"&amp;G13,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I13" s="10" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="10" t="n"/>
+      <c r="H14" s="6">
+        <f>IF(G14="","",HYPERLINK("nota/"&amp;G14,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I14" s="10" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="40" t="n"/>
+      <c r="B15" s="10" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="9" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="10" t="n"/>
+      <c r="H15" s="6">
+        <f>IF(G15="","",HYPERLINK("nota/"&amp;G15,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I15" s="10" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="40" t="n"/>
+      <c r="B16" s="10" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="9" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="6">
+        <f>IF(G16="","",HYPERLINK("nota/"&amp;G16,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I16" s="10" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="40" t="n"/>
+      <c r="B17" s="10" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="9" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="10" t="n"/>
+      <c r="H17" s="6">
+        <f>IF(G17="","",HYPERLINK("nota/"&amp;G17,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I17" s="10" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="41" t="n"/>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Total dana masuk</t>
+        </is>
+      </c>
+      <c r="C18" s="41" t="n"/>
+      <c r="D18" s="13">
+        <f>SUM(D12:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="41" t="n"/>
+      <c r="G18" s="41" t="n"/>
+      <c r="H18" s="41" t="n"/>
+      <c r="I18" s="41" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>2. PENGELUARAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Tanggal</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Barang / keperluan</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Jumlah</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Harga satuan</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Toko</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>File nota</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="40" t="n"/>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>Sensor flow YF-S401 (S2)</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="9" t="n">
+        <v>42211</v>
+      </c>
+      <c r="E22" s="8">
+        <f>IF(D22="","",IF(C22="",1,C22)*D22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="6">
+        <f>IF(G22="","",HYPERLINK("nota/"&amp;G22,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I22" s="10" t="inlineStr">
+        <is>
+          <t>Untuk uji rugi tekanan zona C</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="40" t="n"/>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Sensor flow YF-S201 (S1)</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="9" t="n">
+        <v>29189</v>
+      </c>
+      <c r="E23" s="8">
+        <f>IF(D23="","",IF(C23="",1,C23)*D23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="10" t="n"/>
+      <c r="H23" s="6">
+        <f>IF(G23="","",HYPERLINK("nota/"&amp;G23,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I23" s="10" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="40" t="n"/>
+      <c r="B24" s="10" t="n"/>
+      <c r="C24" s="10" t="n"/>
+      <c r="D24" s="9" t="n"/>
+      <c r="E24" s="8">
+        <f>IF(D24="","",IF(C24="",1,C24)*D24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="6">
+        <f>IF(G24="","",HYPERLINK("nota/"&amp;G24,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I24" s="10" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="40" t="n"/>
+      <c r="B25" s="10" t="n"/>
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="8">
+        <f>IF(D25="","",IF(C25="",1,C25)*D25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="10" t="n"/>
+      <c r="G25" s="10" t="n"/>
+      <c r="H25" s="6">
+        <f>IF(G25="","",HYPERLINK("nota/"&amp;G25,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I25" s="10" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="40" t="n"/>
+      <c r="B26" s="10" t="n"/>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="9" t="n"/>
+      <c r="E26" s="8">
+        <f>IF(D26="","",IF(C26="",1,C26)*D26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="6">
+        <f>IF(G26="","",HYPERLINK("nota/"&amp;G26,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I26" s="10" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="40" t="n"/>
+      <c r="B27" s="10" t="n"/>
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="9" t="n"/>
+      <c r="E27" s="8">
+        <f>IF(D27="","",IF(C27="",1,C27)*D27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="6">
+        <f>IF(G27="","",HYPERLINK("nota/"&amp;G27,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I27" s="10" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="40" t="n"/>
+      <c r="B28" s="10" t="n"/>
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="9" t="n"/>
+      <c r="E28" s="8">
+        <f>IF(D28="","",IF(C28="",1,C28)*D28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="10" t="n"/>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="6">
+        <f>IF(G28="","",HYPERLINK("nota/"&amp;G28,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I28" s="10" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="40" t="n"/>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="8">
+        <f>IF(D29="","",IF(C29="",1,C29)*D29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+      <c r="H29" s="6">
+        <f>IF(G29="","",HYPERLINK("nota/"&amp;G29,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="40" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="9" t="n"/>
+      <c r="E30" s="8">
+        <f>IF(D30="","",IF(C30="",1,C30)*D30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="6">
+        <f>IF(G30="","",HYPERLINK("nota/"&amp;G30,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I30" s="10" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="40" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="9" t="n"/>
+      <c r="E31" s="8">
+        <f>IF(D31="","",IF(C31="",1,C31)*D31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="10" t="n"/>
+      <c r="G31" s="10" t="n"/>
+      <c r="H31" s="6">
+        <f>IF(G31="","",HYPERLINK("nota/"&amp;G31,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I31" s="10" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="40" t="n"/>
+      <c r="B32" s="10" t="n"/>
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="9" t="n"/>
+      <c r="E32" s="8">
+        <f>IF(D32="","",IF(C32="",1,C32)*D32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="10" t="n"/>
+      <c r="H32" s="6">
+        <f>IF(G32="","",HYPERLINK("nota/"&amp;G32,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I32" s="10" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="40" t="n"/>
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="9" t="n"/>
+      <c r="E33" s="8">
+        <f>IF(D33="","",IF(C33="",1,C33)*D33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="10" t="n"/>
+      <c r="G33" s="10" t="n"/>
+      <c r="H33" s="6">
+        <f>IF(G33="","",HYPERLINK("nota/"&amp;G33,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I33" s="10" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="40" t="n"/>
+      <c r="B34" s="10" t="n"/>
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="9" t="n"/>
+      <c r="E34" s="8">
+        <f>IF(D34="","",IF(C34="",1,C34)*D34)</f>
+        <v/>
+      </c>
+      <c r="F34" s="10" t="n"/>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="6">
+        <f>IF(G34="","",HYPERLINK("nota/"&amp;G34,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I34" s="10" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="40" t="n"/>
+      <c r="B35" s="10" t="n"/>
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="9" t="n"/>
+      <c r="E35" s="8">
+        <f>IF(D35="","",IF(C35="",1,C35)*D35)</f>
+        <v/>
+      </c>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="n"/>
+      <c r="H35" s="6">
+        <f>IF(G35="","",HYPERLINK("nota/"&amp;G35,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I35" s="10" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="40" t="n"/>
+      <c r="B36" s="10" t="n"/>
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="8">
+        <f>IF(D36="","",IF(C36="",1,C36)*D36)</f>
+        <v/>
+      </c>
+      <c r="F36" s="10" t="n"/>
+      <c r="G36" s="10" t="n"/>
+      <c r="H36" s="6">
+        <f>IF(G36="","",HYPERLINK("nota/"&amp;G36,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I36" s="10" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="40" t="n"/>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="8">
+        <f>IF(D37="","",IF(C37="",1,C37)*D37)</f>
+        <v/>
+      </c>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="6">
+        <f>IF(G37="","",HYPERLINK("nota/"&amp;G37,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I37" s="10" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="40" t="n"/>
+      <c r="B38" s="10" t="n"/>
+      <c r="C38" s="10" t="n"/>
+      <c r="D38" s="9" t="n"/>
+      <c r="E38" s="8">
+        <f>IF(D38="","",IF(C38="",1,C38)*D38)</f>
+        <v/>
+      </c>
+      <c r="F38" s="10" t="n"/>
+      <c r="G38" s="10" t="n"/>
+      <c r="H38" s="6">
+        <f>IF(G38="","",HYPERLINK("nota/"&amp;G38,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I38" s="10" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="40" t="n"/>
+      <c r="B39" s="10" t="n"/>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="9" t="n"/>
+      <c r="E39" s="8">
+        <f>IF(D39="","",IF(C39="",1,C39)*D39)</f>
+        <v/>
+      </c>
+      <c r="F39" s="10" t="n"/>
+      <c r="G39" s="10" t="n"/>
+      <c r="H39" s="6">
+        <f>IF(G39="","",HYPERLINK("nota/"&amp;G39,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I39" s="10" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="40" t="n"/>
+      <c r="B40" s="10" t="n"/>
+      <c r="C40" s="10" t="n"/>
+      <c r="D40" s="9" t="n"/>
+      <c r="E40" s="8">
+        <f>IF(D40="","",IF(C40="",1,C40)*D40)</f>
+        <v/>
+      </c>
+      <c r="F40" s="10" t="n"/>
+      <c r="G40" s="10" t="n"/>
+      <c r="H40" s="6">
+        <f>IF(G40="","",HYPERLINK("nota/"&amp;G40,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I40" s="10" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="40" t="n"/>
+      <c r="B41" s="10" t="n"/>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="9" t="n"/>
+      <c r="E41" s="8">
+        <f>IF(D41="","",IF(C41="",1,C41)*D41)</f>
+        <v/>
+      </c>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="10" t="n"/>
+      <c r="H41" s="6">
+        <f>IF(G41="","",HYPERLINK("nota/"&amp;G41,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I41" s="10" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="40" t="n"/>
+      <c r="B42" s="10" t="n"/>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="9" t="n"/>
+      <c r="E42" s="8">
+        <f>IF(D42="","",IF(C42="",1,C42)*D42)</f>
+        <v/>
+      </c>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="6">
+        <f>IF(G42="","",HYPERLINK("nota/"&amp;G42,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I42" s="10" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="40" t="n"/>
+      <c r="B43" s="10" t="n"/>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="9" t="n"/>
+      <c r="E43" s="8">
+        <f>IF(D43="","",IF(C43="",1,C43)*D43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="10" t="n"/>
+      <c r="H43" s="6">
+        <f>IF(G43="","",HYPERLINK("nota/"&amp;G43,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I43" s="10" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="40" t="n"/>
+      <c r="B44" s="10" t="n"/>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="8">
+        <f>IF(D44="","",IF(C44="",1,C44)*D44)</f>
+        <v/>
+      </c>
+      <c r="F44" s="10" t="n"/>
+      <c r="G44" s="10" t="n"/>
+      <c r="H44" s="6">
+        <f>IF(G44="","",HYPERLINK("nota/"&amp;G44,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I44" s="10" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="40" t="n"/>
+      <c r="B45" s="10" t="n"/>
+      <c r="C45" s="10" t="n"/>
+      <c r="D45" s="9" t="n"/>
+      <c r="E45" s="8">
+        <f>IF(D45="","",IF(C45="",1,C45)*D45)</f>
+        <v/>
+      </c>
+      <c r="F45" s="10" t="n"/>
+      <c r="G45" s="10" t="n"/>
+      <c r="H45" s="6">
+        <f>IF(G45="","",HYPERLINK("nota/"&amp;G45,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I45" s="10" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="40" t="n"/>
+      <c r="B46" s="10" t="n"/>
+      <c r="C46" s="10" t="n"/>
+      <c r="D46" s="9" t="n"/>
+      <c r="E46" s="8">
+        <f>IF(D46="","",IF(C46="",1,C46)*D46)</f>
+        <v/>
+      </c>
+      <c r="F46" s="10" t="n"/>
+      <c r="G46" s="10" t="n"/>
+      <c r="H46" s="6">
+        <f>IF(G46="","",HYPERLINK("nota/"&amp;G46,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I46" s="10" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="40" t="n"/>
+      <c r="B47" s="10" t="n"/>
+      <c r="C47" s="10" t="n"/>
+      <c r="D47" s="9" t="n"/>
+      <c r="E47" s="8">
+        <f>IF(D47="","",IF(C47="",1,C47)*D47)</f>
+        <v/>
+      </c>
+      <c r="F47" s="10" t="n"/>
+      <c r="G47" s="10" t="n"/>
+      <c r="H47" s="6">
+        <f>IF(G47="","",HYPERLINK("nota/"&amp;G47,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I47" s="10" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="40" t="n"/>
+      <c r="B48" s="10" t="n"/>
+      <c r="C48" s="10" t="n"/>
+      <c r="D48" s="9" t="n"/>
+      <c r="E48" s="8">
+        <f>IF(D48="","",IF(C48="",1,C48)*D48)</f>
+        <v/>
+      </c>
+      <c r="F48" s="10" t="n"/>
+      <c r="G48" s="10" t="n"/>
+      <c r="H48" s="6">
+        <f>IF(G48="","",HYPERLINK("nota/"&amp;G48,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I48" s="10" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="40" t="n"/>
+      <c r="B49" s="10" t="n"/>
+      <c r="C49" s="10" t="n"/>
+      <c r="D49" s="9" t="n"/>
+      <c r="E49" s="8">
+        <f>IF(D49="","",IF(C49="",1,C49)*D49)</f>
+        <v/>
+      </c>
+      <c r="F49" s="10" t="n"/>
+      <c r="G49" s="10" t="n"/>
+      <c r="H49" s="6">
+        <f>IF(G49="","",HYPERLINK("nota/"&amp;G49,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I49" s="10" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="40" t="n"/>
+      <c r="B50" s="10" t="n"/>
+      <c r="C50" s="10" t="n"/>
+      <c r="D50" s="9" t="n"/>
+      <c r="E50" s="8">
+        <f>IF(D50="","",IF(C50="",1,C50)*D50)</f>
+        <v/>
+      </c>
+      <c r="F50" s="10" t="n"/>
+      <c r="G50" s="10" t="n"/>
+      <c r="H50" s="6">
+        <f>IF(G50="","",HYPERLINK("nota/"&amp;G50,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I50" s="10" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="40" t="n"/>
+      <c r="B51" s="10" t="n"/>
+      <c r="C51" s="10" t="n"/>
+      <c r="D51" s="9" t="n"/>
+      <c r="E51" s="8">
+        <f>IF(D51="","",IF(C51="",1,C51)*D51)</f>
+        <v/>
+      </c>
+      <c r="F51" s="10" t="n"/>
+      <c r="G51" s="10" t="n"/>
+      <c r="H51" s="6">
+        <f>IF(G51="","",HYPERLINK("nota/"&amp;G51,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I51" s="10" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="40" t="n"/>
+      <c r="B52" s="10" t="n"/>
+      <c r="C52" s="10" t="n"/>
+      <c r="D52" s="9" t="n"/>
+      <c r="E52" s="8">
+        <f>IF(D52="","",IF(C52="",1,C52)*D52)</f>
+        <v/>
+      </c>
+      <c r="F52" s="10" t="n"/>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="6">
+        <f>IF(G52="","",HYPERLINK("nota/"&amp;G52,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I52" s="10" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="40" t="n"/>
+      <c r="B53" s="10" t="n"/>
+      <c r="C53" s="10" t="n"/>
+      <c r="D53" s="9" t="n"/>
+      <c r="E53" s="8">
+        <f>IF(D53="","",IF(C53="",1,C53)*D53)</f>
+        <v/>
+      </c>
+      <c r="F53" s="10" t="n"/>
+      <c r="G53" s="10" t="n"/>
+      <c r="H53" s="6">
+        <f>IF(G53="","",HYPERLINK("nota/"&amp;G53,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I53" s="10" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="40" t="n"/>
+      <c r="B54" s="10" t="n"/>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="9" t="n"/>
+      <c r="E54" s="8">
+        <f>IF(D54="","",IF(C54="",1,C54)*D54)</f>
+        <v/>
+      </c>
+      <c r="F54" s="10" t="n"/>
+      <c r="G54" s="10" t="n"/>
+      <c r="H54" s="6">
+        <f>IF(G54="","",HYPERLINK("nota/"&amp;G54,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I54" s="10" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="40" t="n"/>
+      <c r="B55" s="10" t="n"/>
+      <c r="C55" s="10" t="n"/>
+      <c r="D55" s="9" t="n"/>
+      <c r="E55" s="8">
+        <f>IF(D55="","",IF(C55="",1,C55)*D55)</f>
+        <v/>
+      </c>
+      <c r="F55" s="10" t="n"/>
+      <c r="G55" s="10" t="n"/>
+      <c r="H55" s="6">
+        <f>IF(G55="","",HYPERLINK("nota/"&amp;G55,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I55" s="10" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="40" t="n"/>
+      <c r="B56" s="10" t="n"/>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="9" t="n"/>
+      <c r="E56" s="8">
+        <f>IF(D56="","",IF(C56="",1,C56)*D56)</f>
+        <v/>
+      </c>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="6">
+        <f>IF(G56="","",HYPERLINK("nota/"&amp;G56,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I56" s="10" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="40" t="n"/>
+      <c r="B57" s="10" t="n"/>
+      <c r="C57" s="10" t="n"/>
+      <c r="D57" s="9" t="n"/>
+      <c r="E57" s="8">
+        <f>IF(D57="","",IF(C57="",1,C57)*D57)</f>
+        <v/>
+      </c>
+      <c r="F57" s="10" t="n"/>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="6">
+        <f>IF(G57="","",HYPERLINK("nota/"&amp;G57,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I57" s="10" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="40" t="n"/>
+      <c r="B58" s="10" t="n"/>
+      <c r="C58" s="10" t="n"/>
+      <c r="D58" s="9" t="n"/>
+      <c r="E58" s="8">
+        <f>IF(D58="","",IF(C58="",1,C58)*D58)</f>
+        <v/>
+      </c>
+      <c r="F58" s="10" t="n"/>
+      <c r="G58" s="10" t="n"/>
+      <c r="H58" s="6">
+        <f>IF(G58="","",HYPERLINK("nota/"&amp;G58,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I58" s="10" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="40" t="n"/>
+      <c r="B59" s="10" t="n"/>
+      <c r="C59" s="10" t="n"/>
+      <c r="D59" s="9" t="n"/>
+      <c r="E59" s="8">
+        <f>IF(D59="","",IF(C59="",1,C59)*D59)</f>
+        <v/>
+      </c>
+      <c r="F59" s="10" t="n"/>
+      <c r="G59" s="10" t="n"/>
+      <c r="H59" s="6">
+        <f>IF(G59="","",HYPERLINK("nota/"&amp;G59,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I59" s="10" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="40" t="n"/>
+      <c r="B60" s="10" t="n"/>
+      <c r="C60" s="10" t="n"/>
+      <c r="D60" s="9" t="n"/>
+      <c r="E60" s="8">
+        <f>IF(D60="","",IF(C60="",1,C60)*D60)</f>
+        <v/>
+      </c>
+      <c r="F60" s="10" t="n"/>
+      <c r="G60" s="10" t="n"/>
+      <c r="H60" s="6">
+        <f>IF(G60="","",HYPERLINK("nota/"&amp;G60,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I60" s="10" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="40" t="n"/>
+      <c r="B61" s="10" t="n"/>
+      <c r="C61" s="10" t="n"/>
+      <c r="D61" s="9" t="n"/>
+      <c r="E61" s="8">
+        <f>IF(D61="","",IF(C61="",1,C61)*D61)</f>
+        <v/>
+      </c>
+      <c r="F61" s="10" t="n"/>
+      <c r="G61" s="10" t="n"/>
+      <c r="H61" s="6">
+        <f>IF(G61="","",HYPERLINK("nota/"&amp;G61,"buka"))</f>
+        <v/>
+      </c>
+      <c r="I61" s="10" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="41" t="n"/>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>Total pengeluaran</t>
+        </is>
+      </c>
+      <c r="C62" s="41" t="n"/>
+      <c r="D62" s="41" t="n"/>
+      <c r="E62" s="13">
+        <f>SUM(E22:E61)</f>
+        <v/>
+      </c>
+      <c r="F62" s="41" t="n"/>
+      <c r="G62" s="41" t="n"/>
+      <c r="H62" s="41" t="n"/>
+      <c r="I62" s="41" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E28"/>
@@ -6094,13 +7158,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -6207,6 +7271,34 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" s="42" t="inlineStr">
+        <is>
+          <t>KEUANGAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• Sheet Keuangan: catat setiap dana masuk dan setiap pembelian. Sisa dana dihitung otomatis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>• Nota disimpan di folder anggaran/nota/ dengan nama TANGGAL_barang.jpg; tulis nama file di kolom File nota.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>• Setelah membeli, isi juga harga beli dan status 'Diterima' di sheet RAB supaya total RAB memakai harga nyata.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>